<commit_message>
Clean release build warnings
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-16</t>
+17</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-9</t>
+10</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -638,7 +638,7 @@
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Complete
-56%</t>
+59%</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="15">
@@ -1734,7 +1734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1932,13 +1932,39 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
+      <c r="A9" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Release build hygiene</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Keep Release x64 build free of app warnings.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Source-generated settings JSON and trimming disabled.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="n"/>
@@ -2021,11 +2047,20 @@
       <c r="F18" s="11" t="n"/>
       <c r="G18" s="11" t="n"/>
     </row>
+    <row r="19">
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F18">
+  <conditionalFormatting sqref="F5:F19">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2039,7 +2074,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E18">
+  <conditionalFormatting sqref="E5:E19">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2054,10 +2089,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Polish dashboard from generated mockup
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -154,8 +154,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -614,19 +614,19 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-17</t>
+19</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-10</t>
+13</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
           <t>In Progress
-3</t>
+2</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -638,7 +638,7 @@
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Complete
-59%</t>
+68%</t>
         </is>
       </c>
     </row>
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.5</v>
+        <v>0.5714285714285714</v>
       </c>
     </row>
   </sheetData>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -808,7 +808,7 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>Built in WinUI.</t>
+          <t>Refined from generated dashboard reference.</t>
         </is>
       </c>
     </row>
@@ -988,100 +988,135 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
+      <c r="A11" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Dashboard visual polish</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Match Dashboard layout to generated Oxygen Taskbar direction.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Dark shell, KPI cards, opacity rail, segmented actions, and runtime rows.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="n"/>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="11" t="n"/>
-      <c r="G18" s="11" t="n"/>
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="10" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="n"/>
-      <c r="B19" s="10" t="n"/>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="11" t="n"/>
+      <c r="G19" s="11" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n"/>
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="11" t="n"/>
-      <c r="G20" s="11" t="n"/>
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="10" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="11" t="n"/>
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
+      <c r="F21" s="11" t="n"/>
+      <c r="G21" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F20">
+  <conditionalFormatting sqref="F5:F21">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -1095,7 +1130,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E20">
+  <conditionalFormatting sqref="E5:E21">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -1110,10 +1145,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1326,94 +1361,94 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="11" t="n"/>
-      <c r="G10" s="11" t="n"/>
+      <c r="A10" s="10" t="n"/>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="n"/>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="11" t="n"/>
-      <c r="G18" s="11" t="n"/>
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1594,94 +1629,94 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="n"/>
-      <c r="B7" s="10" t="n"/>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n"/>
-      <c r="B8" s="11" t="n"/>
-      <c r="C8" s="11" t="n"/>
-      <c r="D8" s="11" t="n"/>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="11" t="n"/>
-      <c r="G8" s="11" t="n"/>
+      <c r="A8" s="10" t="n"/>
+      <c r="B8" s="10" t="n"/>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="10" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="10" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="11" t="n"/>
-      <c r="G10" s="11" t="n"/>
+      <c r="A10" s="10" t="n"/>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1734,7 +1769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1922,12 +1957,12 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Created/pushed during this pass if network permits.</t>
+          <t>Remote created and main/snapshots pushed.</t>
         </is>
       </c>
     </row>
@@ -1967,100 +2002,135 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="11" t="n"/>
-      <c r="G10" s="11" t="n"/>
+      <c r="A10" s="9" t="n">
+        <v>19</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Self-contained launch</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Launch unpackaged WinUI without requiring registered Windows App Runtime.</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Windows App SDK self-contained settings added and launcher verified.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="n"/>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="11" t="n"/>
-      <c r="G18" s="11" t="n"/>
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="10" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="n"/>
-      <c r="B19" s="10" t="n"/>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="11" t="n"/>
+      <c r="G19" s="11" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F19">
+  <conditionalFormatting sqref="F5:F20">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2074,7 +2144,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E19">
+  <conditionalFormatting sqref="E5:E20">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2089,10 +2159,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add V1 P1 mockup prompts
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -154,8 +154,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -614,19 +614,19 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-19</t>
+20</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-13</t>
+14</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
           <t>In Progress
-2</t>
+3</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -638,7 +638,7 @@
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Complete
-68%</t>
+70%</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.625</v>
       </c>
     </row>
   </sheetData>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -978,12 +978,12 @@
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>Waiting for user-generated images.</t>
+          <t>V1 P1 prompt batch prepared; waiting for user-generated images.</t>
         </is>
       </c>
     </row>
@@ -1023,100 +1023,135 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="A12" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>V1 P1 mockup prompt handoff</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Prompt next batch of supporting app states and edge cases.</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Covers onboarding, customization, monitor detail, automation builder, diagnostics error, hotkeys, tray, and about/update.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="11" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="n"/>
-      <c r="B21" s="11" t="n"/>
-      <c r="C21" s="11" t="n"/>
-      <c r="D21" s="11" t="n"/>
-      <c r="E21" s="11" t="n"/>
-      <c r="F21" s="11" t="n"/>
-      <c r="G21" s="11" t="n"/>
+      <c r="A21" s="10" t="n"/>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="10" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="n"/>
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="11" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="11" t="n"/>
+      <c r="G22" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F21">
+  <conditionalFormatting sqref="F5:F22">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -1130,7 +1165,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E21">
+  <conditionalFormatting sqref="E5:E22">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -1145,10 +1180,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1361,94 +1396,94 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n"/>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n"/>
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="10" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1629,94 +1664,94 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n"/>
-      <c r="B7" s="11" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="11" t="n"/>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="11" t="n"/>
-      <c r="G7" s="11" t="n"/>
+      <c r="A7" s="10" t="n"/>
+      <c r="B7" s="10" t="n"/>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="10" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="n"/>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n"/>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n"/>
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="10" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2037,94 +2072,94 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Organize V1 P1 mockup batch
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -154,8 +154,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -614,19 +614,19 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-21</t>
+22</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-15</t>
+17</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
           <t>In Progress
-3</t>
+2</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
@@ -638,7 +638,7 @@
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Complete
-71%</t>
+77%</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -978,12 +978,12 @@
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>V1 P1 first-run onboarding mockup organized; remaining V1 P1 screens pending.</t>
+          <t>V1 P1 mockup batch organized into logical screen folders.</t>
         </is>
       </c>
     </row>
@@ -1093,100 +1093,135 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="A14" s="9" t="n">
+        <v>22</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>V1 P1 mockup organization</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Organize generated supporting app states and edge cases.</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Presets, monitors, automation, diagnostics, settings, tray, about, and alternate onboarding states organized.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="11" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="n"/>
-      <c r="B21" s="11" t="n"/>
-      <c r="C21" s="11" t="n"/>
-      <c r="D21" s="11" t="n"/>
-      <c r="E21" s="11" t="n"/>
-      <c r="F21" s="11" t="n"/>
-      <c r="G21" s="11" t="n"/>
+      <c r="A21" s="10" t="n"/>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="10" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="n"/>
-      <c r="B22" s="10" t="n"/>
-      <c r="C22" s="10" t="n"/>
-      <c r="D22" s="10" t="n"/>
-      <c r="E22" s="10" t="n"/>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
+      <c r="A22" s="11" t="n"/>
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="11" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="11" t="n"/>
+      <c r="G22" s="11" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n"/>
-      <c r="B23" s="11" t="n"/>
-      <c r="C23" s="11" t="n"/>
-      <c r="D23" s="11" t="n"/>
-      <c r="E23" s="11" t="n"/>
-      <c r="F23" s="11" t="n"/>
-      <c r="G23" s="11" t="n"/>
+      <c r="A23" s="10" t="n"/>
+      <c r="B23" s="10" t="n"/>
+      <c r="C23" s="10" t="n"/>
+      <c r="D23" s="10" t="n"/>
+      <c r="E23" s="10" t="n"/>
+      <c r="F23" s="10" t="n"/>
+      <c r="G23" s="10" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="n"/>
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="11" t="n"/>
+      <c r="G24" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F23">
+  <conditionalFormatting sqref="F5:F24">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -1200,7 +1235,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E23">
+  <conditionalFormatting sqref="E5:E24">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -1215,10 +1250,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1431,94 +1466,94 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n"/>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n"/>
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="10" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1699,94 +1734,94 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n"/>
-      <c r="B7" s="11" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="11" t="n"/>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="11" t="n"/>
-      <c r="G7" s="11" t="n"/>
+      <c r="A7" s="10" t="n"/>
+      <c r="B7" s="10" t="n"/>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="10" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="n"/>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="11" t="n"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n"/>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n"/>
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="10" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2107,94 +2142,94 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Implement V1 P1 screen states
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -154,8 +154,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-22</t>
+24</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-17</t>
+19</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -638,7 +638,7 @@
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Complete
-77%</t>
+79%</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="14">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.8</v>
+        <v>0.8181818181818182</v>
       </c>
     </row>
   </sheetData>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1128,100 +1128,135 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
+      <c r="A15" s="8" t="n">
+        <v>23</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>V1 P1 screen implementation</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Implement supporting app states from the organized V1 P1 mockups.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>First-run, preset editor, monitor detail, rule builder, diagnostics error, hotkeys, and about/update surfaces added.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="n"/>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="11" t="n"/>
-      <c r="G18" s="11" t="n"/>
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="10" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="n"/>
-      <c r="B19" s="10" t="n"/>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="11" t="n"/>
+      <c r="G19" s="11" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n"/>
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="11" t="n"/>
-      <c r="G20" s="11" t="n"/>
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="10" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="n"/>
-      <c r="B21" s="10" t="n"/>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n"/>
-      <c r="E21" s="10" t="n"/>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
+      <c r="A21" s="11" t="n"/>
+      <c r="B21" s="11" t="n"/>
+      <c r="C21" s="11" t="n"/>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
+      <c r="F21" s="11" t="n"/>
+      <c r="G21" s="11" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="n"/>
-      <c r="B22" s="11" t="n"/>
-      <c r="C22" s="11" t="n"/>
-      <c r="D22" s="11" t="n"/>
-      <c r="E22" s="11" t="n"/>
-      <c r="F22" s="11" t="n"/>
-      <c r="G22" s="11" t="n"/>
+      <c r="A22" s="10" t="n"/>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="10" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="n"/>
-      <c r="B23" s="10" t="n"/>
-      <c r="C23" s="10" t="n"/>
-      <c r="D23" s="10" t="n"/>
-      <c r="E23" s="10" t="n"/>
-      <c r="F23" s="10" t="n"/>
-      <c r="G23" s="10" t="n"/>
+      <c r="A23" s="11" t="n"/>
+      <c r="B23" s="11" t="n"/>
+      <c r="C23" s="11" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="11" t="n"/>
+      <c r="G23" s="11" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="n"/>
-      <c r="B24" s="11" t="n"/>
-      <c r="C24" s="11" t="n"/>
-      <c r="D24" s="11" t="n"/>
-      <c r="E24" s="11" t="n"/>
-      <c r="F24" s="11" t="n"/>
-      <c r="G24" s="11" t="n"/>
+      <c r="A24" s="10" t="n"/>
+      <c r="B24" s="10" t="n"/>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="10" t="n"/>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="10" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="n"/>
+      <c r="B25" s="11" t="n"/>
+      <c r="C25" s="11" t="n"/>
+      <c r="D25" s="11" t="n"/>
+      <c r="E25" s="11" t="n"/>
+      <c r="F25" s="11" t="n"/>
+      <c r="G25" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F24">
+  <conditionalFormatting sqref="F5:F25">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -1235,7 +1270,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E24">
+  <conditionalFormatting sqref="E5:E25">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -1250,10 +1285,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1268,7 +1303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1466,100 +1501,135 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
+      <c r="A9" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>First-run setup flow</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Route new installs through a local-only onboarding screen before the dashboard.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Start with Oxygen Clear persists completion and enters the dashboard.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="11" t="n"/>
-      <c r="G10" s="11" t="n"/>
+      <c r="A10" s="10" t="n"/>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="n"/>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="11" t="n"/>
-      <c r="G18" s="11" t="n"/>
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="10" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="11" t="n"/>
+      <c r="G19" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F18">
+  <conditionalFormatting sqref="F5:F19">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -1573,7 +1643,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E18">
+  <conditionalFormatting sqref="E5:E19">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -1588,10 +1658,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1734,94 +1804,94 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="n"/>
-      <c r="B7" s="10" t="n"/>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="11" t="n"/>
+      <c r="E7" s="11" t="n"/>
+      <c r="F7" s="11" t="n"/>
+      <c r="G7" s="11" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n"/>
-      <c r="B8" s="11" t="n"/>
-      <c r="C8" s="11" t="n"/>
-      <c r="D8" s="11" t="n"/>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="11" t="n"/>
-      <c r="G8" s="11" t="n"/>
+      <c r="A8" s="10" t="n"/>
+      <c r="B8" s="10" t="n"/>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="10" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="10" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n"/>
-      <c r="B10" s="11" t="n"/>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="11" t="n"/>
-      <c r="G10" s="11" t="n"/>
+      <c r="A10" s="10" t="n"/>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2142,94 +2212,94 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="A12" s="10" t="n"/>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
-      <c r="G13" s="10" t="n"/>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
+      <c r="A14" s="10" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="10" t="n"/>
-      <c r="D15" s="10" t="n"/>
-      <c r="E15" s="10" t="n"/>
-      <c r="F15" s="10" t="n"/>
-      <c r="G15" s="10" t="n"/>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n"/>
-      <c r="B16" s="11" t="n"/>
-      <c r="C16" s="11" t="n"/>
-      <c r="D16" s="11" t="n"/>
-      <c r="E16" s="11" t="n"/>
-      <c r="F16" s="11" t="n"/>
-      <c r="G16" s="11" t="n"/>
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="n"/>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="11" t="n"/>
-      <c r="G18" s="11" t="n"/>
+      <c r="A18" s="10" t="n"/>
+      <c r="B18" s="10" t="n"/>
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="10" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="n"/>
-      <c r="B19" s="10" t="n"/>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
+      <c r="A19" s="11" t="n"/>
+      <c r="B19" s="11" t="n"/>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="11" t="n"/>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="11" t="n"/>
+      <c r="G19" s="11" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n"/>
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="11" t="n"/>
-      <c r="G20" s="11" t="n"/>
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Add tray startup hotkey behavior
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,31 +614,31 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
+26</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Done
 24</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Done
-19</t>
-        </is>
-      </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
           <t>In Progress
-2</t>
+1</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Not Started
-3</t>
+1</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Complete
-79%</t>
+92%</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="13">
@@ -668,7 +668,7 @@
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.8181818181818182</v>
+        <v>0.9090909090909091</v>
       </c>
     </row>
   </sheetData>
@@ -873,12 +873,12 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>Screen exists; native monitor catalog needs expansion.</t>
+          <t>Native taskbar-backed monitor catalog added.</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Background tray menu and open/apply/exit commands.</t>
+          <t>Background tray menu and open/apply/toggle/settings/exit commands.</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -1456,12 +1456,12 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>Placeholder host avoids WinUI/WinForms conflict.</t>
+          <t>Implemented with Shell_NotifyIcon Win32 host to keep WinUI project shape.</t>
         </is>
       </c>
     </row>
@@ -1491,12 +1491,12 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Defaults preserved in settings.</t>
+          <t>Ctrl+Alt+G and Ctrl+Alt+T register against the WinUI window handle.</t>
         </is>
       </c>
     </row>
@@ -1536,13 +1536,39 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
+      <c r="A10" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Startup registration</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Persist Start with Windows through the current-user Run key.</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Settings toggle writes and removes the OxygenTaskbar startup value.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="n"/>
@@ -1625,11 +1651,20 @@
       <c r="F19" s="11" t="n"/>
       <c r="G19" s="11" t="n"/>
     </row>
+    <row r="20">
+      <c r="A20" s="10" t="n"/>
+      <c r="B20" s="10" t="n"/>
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F19">
+  <conditionalFormatting sqref="F5:F20">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -1643,7 +1678,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E19">
+  <conditionalFormatting sqref="E5:E20">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -1658,10 +1693,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1676,7 +1711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1804,13 +1839,39 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n"/>
-      <c r="B7" s="11" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="11" t="n"/>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="11" t="n"/>
-      <c r="G7" s="11" t="n"/>
+      <c r="A7" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Monitor catalog expansion</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>Discover taskbar-backed monitor profiles from primary and secondary taskbar windows.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Maps Shell_TrayWnd and Shell_SecondaryTrayWnd windows to monitor device names.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="n"/>
@@ -1893,11 +1954,20 @@
       <c r="F16" s="10" t="n"/>
       <c r="G16" s="10" t="n"/>
     </row>
+    <row r="17">
+      <c r="A17" s="11" t="n"/>
+      <c r="B17" s="11" t="n"/>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="11" t="n"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F16">
+  <conditionalFormatting sqref="F5:F17">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -1911,7 +1981,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E16">
+  <conditionalFormatting sqref="E5:E17">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -1926,10 +1996,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add runtime automation sensors
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -154,8 +154,8 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -614,31 +614,31 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-26</t>
+28</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-24</t>
+28</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
           <t>In Progress
-1</t>
+0</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Not Started
-1</t>
+0</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Complete
-92%</t>
+100%</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.9090909090909091</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -908,12 +908,12 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>Policy model and toggles are present.</t>
+          <t>Runtime sensors now drive desktop, visible, maximized, fullscreen, and hover states.</t>
         </is>
       </c>
     </row>
@@ -1163,100 +1163,135 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>V1 P2 mockup prompt handoff</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Prepare next generated-image part for post-runtime behavior screens.</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Active reference part created for history, calibration, conflicts, recovery, and multi-monitor telemetry states.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="11" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="n"/>
-      <c r="B21" s="11" t="n"/>
-      <c r="C21" s="11" t="n"/>
-      <c r="D21" s="11" t="n"/>
-      <c r="E21" s="11" t="n"/>
-      <c r="F21" s="11" t="n"/>
-      <c r="G21" s="11" t="n"/>
+      <c r="A21" s="10" t="n"/>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="10" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="n"/>
-      <c r="B22" s="10" t="n"/>
-      <c r="C22" s="10" t="n"/>
-      <c r="D22" s="10" t="n"/>
-      <c r="E22" s="10" t="n"/>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
+      <c r="A22" s="11" t="n"/>
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="11" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="11" t="n"/>
+      <c r="G22" s="11" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n"/>
-      <c r="B23" s="11" t="n"/>
-      <c r="C23" s="11" t="n"/>
-      <c r="D23" s="11" t="n"/>
-      <c r="E23" s="11" t="n"/>
-      <c r="F23" s="11" t="n"/>
-      <c r="G23" s="11" t="n"/>
+      <c r="A23" s="10" t="n"/>
+      <c r="B23" s="10" t="n"/>
+      <c r="C23" s="10" t="n"/>
+      <c r="D23" s="10" t="n"/>
+      <c r="E23" s="10" t="n"/>
+      <c r="F23" s="10" t="n"/>
+      <c r="G23" s="10" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="n"/>
-      <c r="B24" s="10" t="n"/>
-      <c r="C24" s="10" t="n"/>
-      <c r="D24" s="10" t="n"/>
-      <c r="E24" s="10" t="n"/>
-      <c r="F24" s="10" t="n"/>
-      <c r="G24" s="10" t="n"/>
+      <c r="A24" s="11" t="n"/>
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="11" t="n"/>
+      <c r="G24" s="11" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n"/>
-      <c r="B25" s="11" t="n"/>
-      <c r="C25" s="11" t="n"/>
-      <c r="D25" s="11" t="n"/>
-      <c r="E25" s="11" t="n"/>
-      <c r="F25" s="11" t="n"/>
-      <c r="G25" s="11" t="n"/>
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="10" t="n"/>
+      <c r="E25" s="10" t="n"/>
+      <c r="F25" s="10" t="n"/>
+      <c r="G25" s="10" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="n"/>
+      <c r="B26" s="11" t="n"/>
+      <c r="C26" s="11" t="n"/>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="11" t="n"/>
+      <c r="F26" s="11" t="n"/>
+      <c r="G26" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F25">
+  <conditionalFormatting sqref="F5:F26">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -1270,7 +1305,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E25">
+  <conditionalFormatting sqref="E5:E26">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -1285,10 +1320,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1571,94 +1606,94 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1711,7 +1746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1819,7 +1854,7 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Detect active window and fullscreen overlap.</t>
+          <t>Detect active window, maximized, fullscreen, and hover taskbar states.</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -1829,12 +1864,12 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>Policy hooks exist.</t>
+          <t>Win32 foreground, monitor, taskbar, and cursor sensors apply policy on state changes.</t>
         </is>
       </c>
     </row>
@@ -1874,100 +1909,135 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="n"/>
-      <c r="B8" s="10" t="n"/>
-      <c r="C8" s="10" t="n"/>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
+      <c r="A8" s="9" t="n">
+        <v>27</v>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Runtime automation sensors</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Continuously classify runtime desktop/window/fullscreen/hover state.</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Timer-backed sensor applies policy only when the resolved trigger changes.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n"/>
-      <c r="B9" s="11" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n"/>
+      <c r="A9" s="10" t="n"/>
+      <c r="B9" s="10" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="n"/>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F17">
+  <conditionalFormatting sqref="F5:F18">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -1981,7 +2051,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E17">
+  <conditionalFormatting sqref="E5:E18">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -1996,10 +2066,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2282,94 +2352,94 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n"/>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="n"/>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+      <c r="G13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="n"/>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="A15" s="10" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+      <c r="G15" s="10" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="A17" s="10" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="A18" s="11" t="n"/>
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="A20" s="11" t="n"/>
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Add runtime sensor dashboard history
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-28</t>
+34</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-28</t>
+30</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -632,13 +632,13 @@
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Not Started
-0</t>
+4</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Complete
-100%</t>
+88%</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>1</v>
+        <v>0.7777777777777778</v>
       </c>
     </row>
   </sheetData>
@@ -720,7 +720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1198,58 +1198,214 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="n"/>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="n"/>
-      <c r="G17" s="10" t="n"/>
+      <c r="A17" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>V1 P2 mockup organization</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Organize generated post-runtime behavior screens.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>History, calibration, conflict, diagnostics, monitor, settings, and dashboard mockups organized.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="n"/>
-      <c r="B18" s="11" t="n"/>
-      <c r="C18" s="11" t="n"/>
-      <c r="D18" s="11" t="n"/>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="11" t="n"/>
-      <c r="G18" s="11" t="n"/>
+      <c r="A18" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Runtime dashboard implementation</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Implement Dashboard runtime sensor active state from V1 P2.</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard shows active sensor, resolved opacity, automation status, and recent runtime history.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="n"/>
-      <c r="B19" s="10" t="n"/>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
+      <c r="A19" s="8" t="n">
+        <v>31</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Automation history and calibration</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Implement live history, sensor calibration, and conflict warning states.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Mockups organized under Automation.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="n"/>
-      <c r="B20" s="11" t="n"/>
-      <c r="C20" s="11" t="n"/>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
-      <c r="F20" s="11" t="n"/>
-      <c r="G20" s="11" t="n"/>
+      <c r="A20" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Diagnostics recovery states</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Implement sensor timeline and hotkey conflict recovery views.</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Mockups organized under Diagnostics.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="n"/>
-      <c r="B21" s="10" t="n"/>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n"/>
-      <c r="E21" s="10" t="n"/>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
+      <c r="A21" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Multi-display overview</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Implement monitor overview with multi-display state and recent actions.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Mockup organized under Monitors.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="n"/>
-      <c r="B22" s="11" t="n"/>
-      <c r="C22" s="11" t="n"/>
-      <c r="D22" s="11" t="n"/>
-      <c r="E22" s="11" t="n"/>
-      <c r="F22" s="11" t="n"/>
-      <c r="G22" s="11" t="n"/>
+      <c r="A22" s="9" t="n">
+        <v>34</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Startup permission warning</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Implement startup registration failure recovery state.</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>Mockup organized under Settings.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n"/>
@@ -1287,11 +1443,65 @@
       <c r="F26" s="11" t="n"/>
       <c r="G26" s="11" t="n"/>
     </row>
+    <row r="27">
+      <c r="A27" s="10" t="n"/>
+      <c r="B27" s="10" t="n"/>
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="10" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="10" t="n"/>
+      <c r="G27" s="10" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="n"/>
+      <c r="B28" s="11" t="n"/>
+      <c r="C28" s="11" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="11" t="n"/>
+      <c r="G28" s="11" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="n"/>
+      <c r="B29" s="10" t="n"/>
+      <c r="C29" s="10" t="n"/>
+      <c r="D29" s="10" t="n"/>
+      <c r="E29" s="10" t="n"/>
+      <c r="F29" s="10" t="n"/>
+      <c r="G29" s="10" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="n"/>
+      <c r="B30" s="11" t="n"/>
+      <c r="C30" s="11" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="11" t="n"/>
+      <c r="G30" s="11" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n"/>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="10" t="n"/>
+      <c r="E31" s="10" t="n"/>
+      <c r="F31" s="10" t="n"/>
+      <c r="G31" s="10" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="n"/>
+      <c r="B32" s="11" t="n"/>
+      <c r="C32" s="11" t="n"/>
+      <c r="D32" s="11" t="n"/>
+      <c r="E32" s="11" t="n"/>
+      <c r="F32" s="11" t="n"/>
+      <c r="G32" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F26">
+  <conditionalFormatting sqref="F5:F32">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -1305,7 +1515,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E26">
+  <conditionalFormatting sqref="E5:E32">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -1320,10 +1530,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add automation history calibration state
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -620,7 +620,7 @@
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-30</t>
+31</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -632,13 +632,13 @@
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Not Started
-4</t>
+3</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Complete
-88%</t>
+91%</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
   </sheetData>
@@ -1293,12 +1293,12 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Mockups organized under Automation.</t>
+          <t>Automation page shows runtime history, hover calibration, sensor status, and paused-rule recovery.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add diagnostics recovery views
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -620,7 +620,7 @@
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-31</t>
+32</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -632,13 +632,13 @@
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Not Started
-3</t>
+2</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Complete
-91%</t>
+94%</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.8888888888888888</v>
       </c>
     </row>
   </sheetData>
@@ -1328,12 +1328,12 @@
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>Mockups organized under Diagnostics.</t>
+          <t>Diagnostics shows sensor timeline, hotkey status, and reset recovery alongside runtime details.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add monitor overview telemetry
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -620,7 +620,7 @@
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-32</t>
+33</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -632,13 +632,13 @@
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Not Started
-2</t>
+1</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Complete
-94%</t>
+97%</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.9444444444444444</v>
       </c>
     </row>
   </sheetData>
@@ -1363,12 +1363,12 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>Mockup organized under Monitors.</t>
+          <t>Monitor page shows display KPIs, detected display rows, sync state, and recent monitor actions.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add startup recovery warning
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -620,7 +620,7 @@
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-33</t>
+34</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -632,13 +632,13 @@
       <c r="J6" s="3" t="inlineStr">
         <is>
           <t>Not Started
-1</t>
+0</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Complete
-97%</t>
+100%</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.9444444444444444</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1398,12 +1398,12 @@
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>Mockup organized under Settings.</t>
+          <t>Settings shows startup registration status, permission warning copy, and retry recovery.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fade whole taskbar window
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-34</t>
+35</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-34</t>
+35</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1548,7 +1548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1816,13 +1816,39 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
+      <c r="A11" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Whole taskbar transparency parity</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Match old repo behavior by fading taskbar windows and icons, not only accent material.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Taskbar interop now applies WS_EX_LAYERED and SetLayeredWindowAttributes after material composition.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="n"/>
@@ -1905,11 +1931,20 @@
       <c r="F20" s="11" t="n"/>
       <c r="G20" s="11" t="n"/>
     </row>
+    <row r="21">
+      <c r="A21" s="10" t="n"/>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F20">
+  <conditionalFormatting sqref="F5:F21">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -1923,7 +1958,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E20">
+  <conditionalFormatting sqref="E5:E21">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -1938,10 +1973,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add fade transition controls
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-35</t>
+36</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-35</t>
+36</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1548,7 +1548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1851,13 +1851,39 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
+      <c r="A12" s="9" t="n">
+        <v>36</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
+          <t>Fade transition controls</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Expose fade duration and easing settings and animate taskbar opacity changes.</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>Presets now save fade speed/easing and taskbar alpha changes animate with cancellable easing.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="n"/>
@@ -1940,11 +1966,20 @@
       <c r="F21" s="10" t="n"/>
       <c r="G21" s="10" t="n"/>
     </row>
+    <row r="22">
+      <c r="A22" s="11" t="n"/>
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="11" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="11" t="n"/>
+      <c r="G22" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F21">
+  <conditionalFormatting sqref="F5:F22">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -1958,7 +1993,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E21">
+  <conditionalFormatting sqref="E5:E22">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -1973,10 +2008,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Migrate transition timing settings
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-37</t>
+38</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-37</t>
+38</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -2399,7 +2399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2667,13 +2667,39 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
+      <c r="A11" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Transition settings migration</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Preserve existing fade timing when loading settings created before fade-in/out split.</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Legacy profiles with fadeMilliseconds now hydrate fade-in and fade-out instead of becoming instant.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="n"/>
@@ -2756,11 +2782,20 @@
       <c r="F20" s="11" t="n"/>
       <c r="G20" s="11" t="n"/>
     </row>
+    <row r="21">
+      <c r="A21" s="10" t="n"/>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F20">
+  <conditionalFormatting sqref="F5:F21">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2774,7 +2809,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E20">
+  <conditionalFormatting sqref="E5:E21">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2789,10 +2824,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix tuning save profile preservation
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-38</t>
+39</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-38</t>
+39</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -823,12 +823,12 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Presets</t>
+          <t>Tuning</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Material preset selection screen.</t>
+          <t>Material and user settings tuning screen.</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>Clear, Glass, Solid presets.</t>
+          <t>Clear, Glass, Solid presets plus transition, sensor, startup, tray, and hotkey settings.</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>Settings shows startup registration status, permission warning copy, and retry recovery.</t>
+          <t>Tuning shows startup registration status, permission warning copy, and retry recovery.</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>Presets now save fade speed/easing and taskbar alpha changes animate with cancellable easing.</t>
+          <t>Tuning now saves fade speed/easing and taskbar alpha changes animate with cancellable easing.</t>
         </is>
       </c>
     </row>
@@ -1921,13 +1921,39 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n"/>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="11" t="n"/>
-      <c r="E14" s="11" t="n"/>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="11" t="n"/>
+      <c r="A14" s="9" t="n">
+        <v>39</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Tuning save edge cases</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Ensure Save changes preserves the active material and visible profile values.</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>Saving from Oxygen Clear no longer silently rebuilds the profile from Focus Glass; blank names preserve the current profile name.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="n"/>
@@ -2010,11 +2036,20 @@
       <c r="F23" s="10" t="n"/>
       <c r="G23" s="10" t="n"/>
     </row>
+    <row r="24">
+      <c r="A24" s="11" t="n"/>
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="11" t="n"/>
+      <c r="G24" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F23">
+  <conditionalFormatting sqref="F5:F24">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2028,7 +2063,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E23">
+  <conditionalFormatting sqref="E5:E24">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2043,10 +2078,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2487,7 +2522,7 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>8 tests passing.</t>
+          <t>Profile migration, tuning, appearance, sensors, hotkeys, policy, and snapshot tests covered.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use tuning hover proximity in sensors
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-39</t>
+40</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-39</t>
+40</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -2096,7 +2096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2294,13 +2294,39 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
+      <c r="A9" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Hover proximity calibration</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Ensure the Tuning hover proximity control drives runtime hover detection.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Runtime sensor now uses the saved hover distance instead of a hard-coded 10 px threshold, with boundary coverage.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="n"/>
@@ -2383,11 +2409,20 @@
       <c r="F18" s="11" t="n"/>
       <c r="G18" s="11" t="n"/>
     </row>
+    <row r="19">
+      <c r="A19" s="10" t="n"/>
+      <c r="B19" s="10" t="n"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F18">
+  <conditionalFormatting sqref="F5:F19">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2401,7 +2436,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E18">
+  <conditionalFormatting sqref="E5:E19">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2416,10 +2451,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Report hotkey registration status
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-42</t>
+43</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-42</t>
+43</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2026,13 +2026,39 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="9" t="n">
+        <v>43</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Hotkey registration diagnostics</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Report actual Windows hotkey registration success instead of only validating shortcut text.</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Diagnostics now distinguishes registered shortcuts, invalid formats, and Windows registration failures with error codes.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="n"/>
@@ -2115,11 +2141,20 @@
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="11" t="n"/>
     </row>
+    <row r="26">
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="10" t="n"/>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="10" t="n"/>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F25">
+  <conditionalFormatting sqref="F5:F26">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2133,7 +2168,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E25">
+  <conditionalFormatting sqref="E5:E26">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2148,10 +2183,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Cover tray command dispatch
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-43</t>
+44</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-43</t>
+44</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2061,13 +2061,39 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="A17" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Tray command dispatch audit</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Verify tray menu labels and command routing for dashboard, tuning, apply, toggle, and exit.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Tray command labels and dispatch are covered by focused tests; live hidden-window validation confirmed background toggle and dashboard restore outcomes.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n"/>
@@ -2150,11 +2176,20 @@
       <c r="F26" s="10" t="n"/>
       <c r="G26" s="10" t="n"/>
     </row>
+    <row r="27">
+      <c r="A27" s="11" t="n"/>
+      <c r="B27" s="11" t="n"/>
+      <c r="C27" s="11" t="n"/>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="11" t="n"/>
+      <c r="G27" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F26">
+  <conditionalFormatting sqref="F5:F27">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2168,7 +2203,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E26">
+  <conditionalFormatting sqref="E5:E27">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2183,10 +2218,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Preserve tuning profile name edits
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-45</t>
+46</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-45</t>
+46</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2096,13 +2096,39 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="A18" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Tuning profile name edit stability</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Preserve unsaved profile name edits while other Tuning settings refresh.</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Tuning no longer overwrites dirty preset-name input during state refresh; Computer Use reproduced the bug and verified save plus relaunch on a 3440-wide monitor.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="n"/>
@@ -2185,11 +2211,20 @@
       <c r="F27" s="11" t="n"/>
       <c r="G27" s="11" t="n"/>
     </row>
+    <row r="28">
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F27">
+  <conditionalFormatting sqref="F5:F28">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2203,7 +2238,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E27">
+  <conditionalFormatting sqref="E5:E28">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2218,10 +2253,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix tuning material controls
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-46</t>
+47</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-46</t>
+47</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2131,13 +2131,39 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="A19" s="8" t="n">
+        <v>47</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Tuning material and reset edge cases</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Ensure material buttons and Reset behave intentionally from the Tuning screen.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Clear, Acrylic, Mica, and Solid are wired; material changes preserve current tuning values; Reset restores Oxygen Clear; Computer Use verified Solid persistence and Reset on a 3440-wide monitor.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n"/>
@@ -2220,11 +2246,20 @@
       <c r="F28" s="10" t="n"/>
       <c r="G28" s="10" t="n"/>
     </row>
+    <row r="29">
+      <c r="A29" s="11" t="n"/>
+      <c r="B29" s="11" t="n"/>
+      <c r="C29" s="11" t="n"/>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="11" t="n"/>
+      <c r="G29" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F28">
+  <conditionalFormatting sqref="F5:F29">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2238,7 +2273,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E28">
+  <conditionalFormatting sqref="E5:E29">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2253,10 +2288,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Preserve tuning slider edits
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -606,7 +606,7 @@
     <row r="4">
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>LAST_UPDATED: 2026-06-07</t>
+          <t>LAST_UPDATED: 2026-06-08</t>
         </is>
       </c>
     </row>
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-47</t>
+48</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-47</t>
+48</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2166,13 +2166,39 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="A20" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Tuning slider refresh stability</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Preserve unsaved opacity, fade, and easing edits while other Tuning settings refresh.</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Computer Use reproduced hover proximity refresh wiping dirty opacity/fade edits, then verified the dirty tuning values survive on a 3440-wide monitor.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n"/>
@@ -2255,11 +2281,20 @@
       <c r="F29" s="11" t="n"/>
       <c r="G29" s="11" t="n"/>
     </row>
+    <row r="30">
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F29">
+  <conditionalFormatting sqref="F5:F30">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2273,7 +2308,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E29">
+  <conditionalFormatting sqref="E5:E30">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2288,10 +2323,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reset transparency toggle baseline
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-48</t>
+49</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-48</t>
+49</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2201,13 +2201,39 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="n"/>
-      <c r="B21" s="11" t="n"/>
-      <c r="C21" s="11" t="n"/>
-      <c r="D21" s="11" t="n"/>
-      <c r="E21" s="11" t="n"/>
-      <c r="F21" s="11" t="n"/>
-      <c r="G21" s="11" t="n"/>
+      <c r="A21" s="8" t="n">
+        <v>49</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Transparency toggle baseline stability</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Reset stale transparency-toggle restore state when the user applies a new profile or explicit opacity.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>Computer Use reproduced Night Solid inheriting an old 32% toggle baseline after a transparent state, then verified profile changes establish a fresh toggle baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n"/>
@@ -2290,11 +2316,20 @@
       <c r="F30" s="10" t="n"/>
       <c r="G30" s="10" t="n"/>
     </row>
+    <row r="31">
+      <c r="A31" s="11" t="n"/>
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="11" t="n"/>
+      <c r="G31" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F30">
+  <conditionalFormatting sqref="F5:F31">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2308,7 +2343,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E30">
+  <conditionalFormatting sqref="E5:E31">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2323,10 +2358,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix automation policy preview
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-49</t>
+50</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-49</t>
+50</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2236,13 +2236,39 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="n"/>
-      <c r="B22" s="10" t="n"/>
-      <c r="C22" s="10" t="n"/>
-      <c r="D22" s="10" t="n"/>
-      <c r="E22" s="10" t="n"/>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
+      <c r="A22" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Automation policy preview accuracy</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Show actual automation rule targets and live runtime preview instead of static mock values.</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>Computer Use reproduced the 72/85/60/42/Hidden mismatch and verified policy-driven values on a 3440-wide monitor.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n"/>
@@ -2325,11 +2351,20 @@
       <c r="F31" s="11" t="n"/>
       <c r="G31" s="11" t="n"/>
     </row>
+    <row r="32">
+      <c r="A32" s="10" t="n"/>
+      <c r="B32" s="10" t="n"/>
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="10" t="n"/>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="10" t="n"/>
+      <c r="G32" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F31">
+  <conditionalFormatting sqref="F5:F32">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2343,7 +2378,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E31">
+  <conditionalFormatting sqref="E5:E32">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2358,10 +2393,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Enable automation paused recovery
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-50</t>
+51</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-50</t>
+51</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2271,13 +2271,39 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n"/>
-      <c r="B23" s="11" t="n"/>
-      <c r="C23" s="11" t="n"/>
-      <c r="D23" s="11" t="n"/>
-      <c r="E23" s="11" t="n"/>
-      <c r="F23" s="11" t="n"/>
-      <c r="G23" s="11" t="n"/>
+      <c r="A23" s="8" t="n">
+        <v>51</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Automation paused recovery</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Let the Automation conflict card re-enable paused automation directly.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Computer Use reproduced the disabled paused-state recovery button and verified Enable automation now restores live automation on a 3440-wide monitor.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n"/>
@@ -2360,11 +2386,20 @@
       <c r="F32" s="10" t="n"/>
       <c r="G32" s="10" t="n"/>
     </row>
+    <row r="33">
+      <c r="A33" s="11" t="n"/>
+      <c r="B33" s="11" t="n"/>
+      <c r="C33" s="11" t="n"/>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="11" t="n"/>
+      <c r="F33" s="11" t="n"/>
+      <c r="G33" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F32">
+  <conditionalFormatting sqref="F5:F33">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2378,7 +2413,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E32">
+  <conditionalFormatting sqref="E5:E33">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2393,10 +2428,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix diagnostics recovery actions
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-51</t>
+52</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-51</t>
+52</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2306,13 +2306,39 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="n"/>
-      <c r="B24" s="10" t="n"/>
-      <c r="C24" s="10" t="n"/>
-      <c r="D24" s="10" t="n"/>
-      <c r="E24" s="10" t="n"/>
-      <c r="F24" s="10" t="n"/>
-      <c r="G24" s="10" t="n"/>
+      <c r="A24" s="9" t="n">
+        <v>52</v>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Diagnostics recovery action accuracy</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Keep Diagnostics recovery controls truthful and non-destructive.</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>Computer Use reproduced the inert Open folder button, misleading error header, and fullscreen Apply defaults behavior; Diagnostics now opens logs, reports healthy taskbar updates, and applies safe desktop without changing saved settings.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="n"/>
@@ -2395,11 +2421,20 @@
       <c r="F33" s="11" t="n"/>
       <c r="G33" s="11" t="n"/>
     </row>
+    <row r="34">
+      <c r="A34" s="10" t="n"/>
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="10" t="n"/>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="10" t="n"/>
+      <c r="G34" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F33">
+  <conditionalFormatting sqref="F5:F34">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2413,7 +2448,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E33">
+  <conditionalFormatting sqref="E5:E34">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2428,10 +2463,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Enable tuning hotkey edits
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-52</t>
+53</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-52</t>
+53</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2341,13 +2341,39 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n"/>
-      <c r="B25" s="11" t="n"/>
-      <c r="C25" s="11" t="n"/>
-      <c r="D25" s="11" t="n"/>
-      <c r="E25" s="11" t="n"/>
-      <c r="F25" s="11" t="n"/>
-      <c r="G25" s="11" t="n"/>
+      <c r="A25" s="8" t="n">
+        <v>53</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Tuning hotkey editing</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Make the unified Tuning hotkey fields actually editable and persist them through Windows hotkey registration.</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>Computer Use reproduced read-only hotkey fields on the Tuning page; Save changes now writes and re-registers edited shortcuts without overwriting opacity or transition values, with initialization guards added to live-control pages.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n"/>
@@ -2430,11 +2456,20 @@
       <c r="F34" s="10" t="n"/>
       <c r="G34" s="10" t="n"/>
     </row>
+    <row r="35">
+      <c r="A35" s="11" t="n"/>
+      <c r="B35" s="11" t="n"/>
+      <c r="C35" s="11" t="n"/>
+      <c r="D35" s="11" t="n"/>
+      <c r="E35" s="11" t="n"/>
+      <c r="F35" s="11" t="n"/>
+      <c r="G35" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F34">
+  <conditionalFormatting sqref="F5:F35">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2448,7 +2483,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E34">
+  <conditionalFormatting sqref="E5:E35">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2463,10 +2498,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Make settings hotkey status truthful
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-53</t>
+54</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-53</t>
+54</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2376,13 +2376,39 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="n"/>
-      <c r="B26" s="10" t="n"/>
-      <c r="C26" s="10" t="n"/>
-      <c r="D26" s="10" t="n"/>
-      <c r="E26" s="10" t="n"/>
-      <c r="F26" s="10" t="n"/>
-      <c r="G26" s="10" t="n"/>
+      <c r="A26" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Settings hotkey warning accuracy</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Keep the legacy Settings hotkey status truthful if the surface is reached.</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>Replaced the always-visible shortcut conflict warning with the same real Windows registration state used by Diagnostics.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n"/>
@@ -2465,11 +2491,20 @@
       <c r="F35" s="11" t="n"/>
       <c r="G35" s="11" t="n"/>
     </row>
+    <row r="36">
+      <c r="A36" s="10" t="n"/>
+      <c r="B36" s="10" t="n"/>
+      <c r="C36" s="10" t="n"/>
+      <c r="D36" s="10" t="n"/>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F35">
+  <conditionalFormatting sqref="F5:F36">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2483,7 +2518,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E35">
+  <conditionalFormatting sqref="E5:E36">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2498,10 +2533,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Refresh mockup handoff documentation
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-54</t>
+55</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-54</t>
+55</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -2924,7 +2924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3262,13 +3262,39 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n"/>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
+      <c r="A13" s="8" t="n">
+        <v>55</v>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Mockup handoff documentation freshness</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Remove stale active-prompt claims after generated mockups are organized.</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Computer Use swept the live app surfaces, then README and walkthrough were updated so V1 P2 prompt handoff is no longer described as active.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n"/>
@@ -3351,11 +3377,20 @@
       <c r="F22" s="10" t="n"/>
       <c r="G22" s="10" t="n"/>
     </row>
+    <row r="23">
+      <c r="A23" s="11" t="n"/>
+      <c r="B23" s="11" t="n"/>
+      <c r="C23" s="11" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="11" t="n"/>
+      <c r="G23" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F22">
+  <conditionalFormatting sqref="F5:F23">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -3369,7 +3404,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E22">
+  <conditionalFormatting sqref="E5:E23">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -3384,10 +3419,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Clarify automation preview affordances
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-55</t>
+56</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-55</t>
+56</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2411,13 +2411,39 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="n"/>
-      <c r="B27" s="11" t="n"/>
-      <c r="C27" s="11" t="n"/>
-      <c r="D27" s="11" t="n"/>
-      <c r="E27" s="11" t="n"/>
-      <c r="F27" s="11" t="n"/>
-      <c r="G27" s="11" t="n"/>
+      <c r="A27" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Automation preview affordance clarity</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Make Automation read like an intentional policy preview instead of a disabled editor.</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Computer Use reproduced disabled Add custom rule, reset, discard, and save controls; Automation now uses read-only policy output with an active Open Tuning edit path.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n"/>
@@ -2500,11 +2526,20 @@
       <c r="F36" s="10" t="n"/>
       <c r="G36" s="10" t="n"/>
     </row>
+    <row r="37">
+      <c r="A37" s="11" t="n"/>
+      <c r="B37" s="11" t="n"/>
+      <c r="C37" s="11" t="n"/>
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="11" t="n"/>
+      <c r="G37" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F36">
+  <conditionalFormatting sqref="F5:F37">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2518,7 +2553,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E36">
+  <conditionalFormatting sqref="E5:E37">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2533,10 +2568,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Make diagnostics recovery state-aware
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-56</t>
+57</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-56</t>
+57</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2446,13 +2446,39 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="n"/>
-      <c r="B28" s="10" t="n"/>
-      <c r="C28" s="10" t="n"/>
-      <c r="D28" s="10" t="n"/>
-      <c r="E28" s="10" t="n"/>
-      <c r="F28" s="10" t="n"/>
-      <c r="G28" s="10" t="n"/>
+      <c r="A28" s="9" t="n">
+        <v>57</v>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Diagnostics recovery card state</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Keep the Diagnostics recovery card aligned with healthy versus failed taskbar detection.</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>Computer Use found a healthy Diagnostics page still showing probable failure causes; recovery copy is now state-aware and tested.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="n"/>
@@ -2535,11 +2561,20 @@
       <c r="F37" s="11" t="n"/>
       <c r="G37" s="11" t="n"/>
     </row>
+    <row r="38">
+      <c r="A38" s="10" t="n"/>
+      <c r="B38" s="10" t="n"/>
+      <c r="C38" s="10" t="n"/>
+      <c r="D38" s="10" t="n"/>
+      <c r="E38" s="10" t="n"/>
+      <c r="F38" s="10" t="n"/>
+      <c r="G38" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F37">
+  <conditionalFormatting sqref="F5:F38">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2553,7 +2588,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E37">
+  <conditionalFormatting sqref="E5:E38">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2568,10 +2603,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Make about page snapshot-aware
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-57</t>
+58</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-57</t>
+58</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2481,13 +2481,39 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="n"/>
-      <c r="B29" s="11" t="n"/>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="11" t="n"/>
-      <c r="E29" s="11" t="n"/>
-      <c r="F29" s="11" t="n"/>
-      <c r="G29" s="11" t="n"/>
+      <c r="A29" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>About page version and utility actions</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Keep About version labels and utility buttons truthful for local snapshot builds.</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Computer Use found hard-coded 1.0.0 version labels and inert utility buttons; About now reads assembly metadata, opens logs/settings, and reports snapshot update status.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n"/>
@@ -2570,11 +2596,20 @@
       <c r="F38" s="10" t="n"/>
       <c r="G38" s="10" t="n"/>
     </row>
+    <row r="39">
+      <c r="A39" s="11" t="n"/>
+      <c r="B39" s="11" t="n"/>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="11" t="n"/>
+      <c r="G39" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F38">
+  <conditionalFormatting sqref="F5:F39">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2588,7 +2623,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E38">
+  <conditionalFormatting sqref="E5:E39">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2603,10 +2638,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Persist monitor override changes
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-58</t>
+59</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-58</t>
+59</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2516,13 +2516,39 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="n"/>
-      <c r="B30" s="10" t="n"/>
-      <c r="C30" s="10" t="n"/>
-      <c r="D30" s="10" t="n"/>
-      <c r="E30" s="10" t="n"/>
-      <c r="F30" s="10" t="n"/>
-      <c r="G30" s="10" t="n"/>
+      <c r="A30" s="9" t="n">
+        <v>59</v>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Monitor override apply persistence</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Make monitor override controls apply to the selected display instead of the global active profile.</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>Computer Use found monitor Apply reverting edited override values and recording a global desktop apply; monitor overrides now persist per display and feed taskbar opacity resolution.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n"/>
@@ -2605,11 +2631,20 @@
       <c r="F39" s="11" t="n"/>
       <c r="G39" s="11" t="n"/>
     </row>
+    <row r="40">
+      <c r="A40" s="10" t="n"/>
+      <c r="B40" s="10" t="n"/>
+      <c r="C40" s="10" t="n"/>
+      <c r="D40" s="10" t="n"/>
+      <c r="E40" s="10" t="n"/>
+      <c r="F40" s="10" t="n"/>
+      <c r="G40" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F39">
+  <conditionalFormatting sqref="F5:F40">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2623,7 +2658,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E39">
+  <conditionalFormatting sqref="E5:E40">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2638,10 +2673,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Honor per-monitor fade directions
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-59</t>
+60</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-59</t>
+60</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2551,13 +2551,39 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="n"/>
-      <c r="B31" s="11" t="n"/>
-      <c r="C31" s="11" t="n"/>
-      <c r="D31" s="11" t="n"/>
-      <c r="E31" s="11" t="n"/>
-      <c r="F31" s="11" t="n"/>
-      <c r="G31" s="11" t="n"/>
+      <c r="A31" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Per-monitor transition direction audit</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Ensure fade-in and fade-out speeds are honored independently when different taskbars change in different directions.</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>Code audit found multi-monitor animation used the first taskbar as the representative duration; each taskbar now selects its own fade direction, while unchanged taskbars skip no-op animation time.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n"/>
@@ -2640,11 +2666,20 @@
       <c r="F40" s="10" t="n"/>
       <c r="G40" s="10" t="n"/>
     </row>
+    <row r="41">
+      <c r="A41" s="11" t="n"/>
+      <c r="B41" s="11" t="n"/>
+      <c r="C41" s="11" t="n"/>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="11" t="n"/>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F40">
+  <conditionalFormatting sqref="F5:F41">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2658,7 +2693,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E40">
+  <conditionalFormatting sqref="E5:E41">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2673,10 +2708,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Audit hover proximity boundaries
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-60</t>
+61</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-60</t>
+61</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2586,13 +2586,39 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="n"/>
-      <c r="B32" s="10" t="n"/>
-      <c r="C32" s="10" t="n"/>
-      <c r="D32" s="10" t="n"/>
-      <c r="E32" s="10" t="n"/>
-      <c r="F32" s="10" t="n"/>
-      <c r="G32" s="10" t="n"/>
+      <c r="A32" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Hover proximity boundary audit</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Verify hover proximity edge settings behave intentionally at 0 px and 48 px.</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>Computer Use verified Tuning accepts and persists 0 px and 48 px hover proximity; sensor tests now lock zero and negative-distance boundary behavior.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="n"/>
@@ -2675,11 +2701,20 @@
       <c r="F41" s="11" t="n"/>
       <c r="G41" s="11" t="n"/>
     </row>
+    <row r="42">
+      <c r="A42" s="10" t="n"/>
+      <c r="B42" s="10" t="n"/>
+      <c r="C42" s="10" t="n"/>
+      <c r="D42" s="10" t="n"/>
+      <c r="E42" s="10" t="n"/>
+      <c r="F42" s="10" t="n"/>
+      <c r="G42" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F41">
+  <conditionalFormatting sqref="F5:F42">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2693,7 +2728,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E41">
+  <conditionalFormatting sqref="E5:E42">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2708,10 +2743,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Unify runtime state labels
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-61</t>
+62</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-61</t>
+62</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2621,13 +2621,39 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="n"/>
-      <c r="B33" s="11" t="n"/>
-      <c r="C33" s="11" t="n"/>
-      <c r="D33" s="11" t="n"/>
-      <c r="E33" s="11" t="n"/>
-      <c r="F33" s="11" t="n"/>
-      <c r="G33" s="11" t="n"/>
+      <c r="A33" s="8" t="n">
+        <v>62</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Runtime state vocabulary consistency</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Keep runtime state labels consistent across Dashboard, Automation, Monitors, and Diagnostics.</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Source audit found Dashboard, Automation, Monitors, and Diagnostics using different names for the same runtime states; pages now share one runtime vocabulary with tests.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n"/>
@@ -2710,11 +2736,20 @@
       <c r="F42" s="10" t="n"/>
       <c r="G42" s="10" t="n"/>
     </row>
+    <row r="43">
+      <c r="A43" s="11" t="n"/>
+      <c r="B43" s="11" t="n"/>
+      <c r="C43" s="11" t="n"/>
+      <c r="D43" s="11" t="n"/>
+      <c r="E43" s="11" t="n"/>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F42">
+  <conditionalFormatting sqref="F5:F43">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2728,7 +2763,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E42">
+  <conditionalFormatting sqref="E5:E43">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2743,10 +2778,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Clarify manual runtime apply actions
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-62</t>
+63</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-62</t>
+63</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2656,13 +2656,39 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="n"/>
-      <c r="B34" s="10" t="n"/>
-      <c r="C34" s="10" t="n"/>
-      <c r="D34" s="10" t="n"/>
-      <c r="E34" s="10" t="n"/>
-      <c r="F34" s="10" t="n"/>
-      <c r="G34" s="10" t="n"/>
+      <c r="A34" s="9" t="n">
+        <v>63</v>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Manual apply semantics clarity</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>Make manual runtime actions describe whether they reapply the current state or simulate a specific state.</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>Audit found Dashboard and tray Apply forced Desktop while Automation preview simulated Visible window; controls now say and do Reapply current state or Simulate visible window explicitly.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="n"/>
@@ -2745,11 +2771,20 @@
       <c r="F43" s="11" t="n"/>
       <c r="G43" s="11" t="n"/>
     </row>
+    <row r="44">
+      <c r="A44" s="10" t="n"/>
+      <c r="B44" s="10" t="n"/>
+      <c r="C44" s="10" t="n"/>
+      <c r="D44" s="10" t="n"/>
+      <c r="E44" s="10" t="n"/>
+      <c r="F44" s="10" t="n"/>
+      <c r="G44" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F43">
+  <conditionalFormatting sqref="F5:F44">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2763,7 +2798,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E43">
+  <conditionalFormatting sqref="E5:E44">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2778,10 +2813,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Validate hidden-window hotkey restore
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-64</t>
+65</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-64</t>
+65</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2721,18 +2721,44 @@
       </c>
       <c r="G35" s="8" t="inlineStr">
         <is>
-          <t>Computer Use closed the Oxygen window; process inspection confirmed TaskbarTransparency stayed alive with no visible main window and ShowTrayIcon enabled. Hidden-window hotkey restore needs a tray/menu-specific validation path.</t>
+          <t>Computer Use closed the Oxygen window; process inspection confirmed TaskbarTransparency stayed alive with no visible main window and ShowTrayIcon enabled.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="n"/>
-      <c r="B36" s="10" t="n"/>
-      <c r="C36" s="10" t="n"/>
-      <c r="D36" s="10" t="n"/>
-      <c r="E36" s="10" t="n"/>
-      <c r="F36" s="10" t="n"/>
-      <c r="G36" s="10" t="n"/>
+      <c r="A36" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Hidden-window hotkey restore audit</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Verify the global open hotkey restores Oxygen after the dashboard has been hidden to tray.</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>Computer Use closed Oxygen to tray on a 1426 by 913 widescreen app surface, sent Ctrl+Alt+G through Windows, and confirmed the Dashboard window returned at the same bounds.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n"/>
@@ -2815,11 +2841,20 @@
       <c r="F45" s="11" t="n"/>
       <c r="G45" s="11" t="n"/>
     </row>
+    <row r="46">
+      <c r="A46" s="10" t="n"/>
+      <c r="B46" s="10" t="n"/>
+      <c r="C46" s="10" t="n"/>
+      <c r="D46" s="10" t="n"/>
+      <c r="E46" s="10" t="n"/>
+      <c r="F46" s="10" t="n"/>
+      <c r="G46" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F45">
+  <conditionalFormatting sqref="F5:F46">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2833,7 +2868,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E45">
+  <conditionalFormatting sqref="E5:E46">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2848,10 +2883,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Validate tray popup commands
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-65</t>
+66</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-65</t>
+66</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1583,7 +1583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2761,13 +2761,39 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="n"/>
-      <c r="B37" s="11" t="n"/>
-      <c r="C37" s="11" t="n"/>
-      <c r="D37" s="11" t="n"/>
-      <c r="E37" s="11" t="n"/>
-      <c r="F37" s="11" t="n"/>
-      <c r="G37" s="11" t="n"/>
+      <c r="A37" s="8" t="n">
+        <v>66</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Features</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Tray popup command audit</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Verify the notification-area popup exposes the intended commands and routes key commands from the hidden tray state.</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Windows tray overflow exposed Oxygen Taskbar; native popup extraction confirmed Open Dashboard, Reapply Current State, Toggle Transparency, Open Tuning, and Exit labels. Open Tuning restored Tuning, and Exit terminated the background process.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n"/>
@@ -2850,11 +2876,20 @@
       <c r="F46" s="10" t="n"/>
       <c r="G46" s="10" t="n"/>
     </row>
+    <row r="47">
+      <c r="A47" s="11" t="n"/>
+      <c r="B47" s="11" t="n"/>
+      <c r="C47" s="11" t="n"/>
+      <c r="D47" s="11" t="n"/>
+      <c r="E47" s="11" t="n"/>
+      <c r="F47" s="11" t="n"/>
+      <c r="G47" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F46">
+  <conditionalFormatting sqref="F5:F47">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -2868,7 +2903,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E46">
+  <conditionalFormatting sqref="E5:E47">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -2883,10 +2918,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Skip redundant taskbar interop applies
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-67</t>
+68</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-67</t>
+68</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3717,13 +3717,39 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n"/>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
+      <c r="A15" s="8" t="n">
+        <v>68</v>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Taskbar interop no-op optimization</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>Avoid redundant native taskbar composition and alpha calls when visual requests are unchanged.</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>Taskbar appearance requests are cached per handle and unchanged layered-alpha requests are skipped, reducing work during rapid controls and repeated applies.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n"/>
@@ -3806,11 +3832,20 @@
       <c r="F24" s="10" t="n"/>
       <c r="G24" s="10" t="n"/>
     </row>
+    <row r="25">
+      <c r="A25" s="11" t="n"/>
+      <c r="B25" s="11" t="n"/>
+      <c r="C25" s="11" t="n"/>
+      <c r="D25" s="11" t="n"/>
+      <c r="E25" s="11" t="n"/>
+      <c r="F25" s="11" t="n"/>
+      <c r="G25" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F24">
+  <conditionalFormatting sqref="F5:F25">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -3824,7 +3859,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E24">
+  <conditionalFormatting sqref="E5:E25">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -3839,10 +3874,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Debounce slider setting persistence
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-68</t>
+69</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-68</t>
+69</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3752,13 +3752,39 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="A16" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>Slider persistence debounce</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Collapse rapid opacity and hover-distance slider bursts into immediate previews plus one settled settings save.</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard opacity and Tuning hover proximity now preview instantly while debouncing durable settings persistence to reduce drag-time disk churn.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="n"/>
@@ -3841,11 +3867,20 @@
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="11" t="n"/>
     </row>
+    <row r="26">
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="10" t="n"/>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="10" t="n"/>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F25">
+  <conditionalFormatting sqref="F5:F26">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -3859,7 +3894,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E25">
+  <conditionalFormatting sqref="E5:E26">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -3874,10 +3909,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Optimize active page refresh work
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-69</t>
+70</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-69</t>
+70</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3787,13 +3787,39 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="n"/>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
+      <c r="A17" s="8" t="n">
+        <v>70</v>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Active page refresh optimization</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Limit global state refresh work to loaded pages and avoid replacing unchanged runtime list sources.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>Dashboard, Tuning, Automation, Monitors, Diagnostics, and Settings now unsubscribe when unloaded; runtime-heavy lists update only when their source signatures change.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n"/>
@@ -3876,11 +3902,20 @@
       <c r="F26" s="10" t="n"/>
       <c r="G26" s="10" t="n"/>
     </row>
+    <row r="27">
+      <c r="A27" s="11" t="n"/>
+      <c r="B27" s="11" t="n"/>
+      <c r="C27" s="11" t="n"/>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="11" t="n"/>
+      <c r="G27" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F26">
+  <conditionalFormatting sqref="F5:F27">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -3894,7 +3929,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E26">
+  <conditionalFormatting sqref="E5:E27">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -3909,10 +3944,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Skip unchanged startup monitor saves
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-70</t>
+71</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-70</t>
+71</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3822,13 +3822,39 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="n"/>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
+      <c r="A18" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Startup monitor refresh no-op guard</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Avoid startup settings writes and live monitor collection resets when detected monitors match saved state.</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Monitor refresh now merges detected display metadata with saved overrides, updates live monitors only when changed, and saves only when the effective monitor list changes.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="n"/>
@@ -3911,11 +3937,20 @@
       <c r="F27" s="11" t="n"/>
       <c r="G27" s="11" t="n"/>
     </row>
+    <row r="28">
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F27">
+  <conditionalFormatting sqref="F5:F28">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -3929,7 +3964,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E27">
+  <conditionalFormatting sqref="E5:E28">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -3944,10 +3979,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Share taskbar window discovery
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-71</t>
+72</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-71</t>
+72</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3857,13 +3857,39 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="n"/>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
+      <c r="A19" s="8" t="n">
+        <v>72</v>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Shared taskbar window discovery</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Centralize native taskbar enumeration and monitor metadata lookup used by sensors, monitor catalog, and appearance apply.</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>TaskbarWindowCatalog now owns Shell_TrayWnd and Shell_SecondaryTrayWnd discovery so services reuse one native lookup path instead of duplicating Win32 enumeration code.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n"/>
@@ -3946,11 +3972,20 @@
       <c r="F28" s="10" t="n"/>
       <c r="G28" s="10" t="n"/>
     </row>
+    <row r="29">
+      <c r="A29" s="11" t="n"/>
+      <c r="B29" s="11" t="n"/>
+      <c r="C29" s="11" t="n"/>
+      <c r="D29" s="11" t="n"/>
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="11" t="n"/>
+      <c r="G29" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F28">
+  <conditionalFormatting sqref="F5:F29">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -3964,7 +3999,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E28">
+  <conditionalFormatting sqref="E5:E29">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -3979,10 +4014,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Clean up taskbar animation caches
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-72</t>
+73</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-72</t>
+73</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3892,13 +3892,39 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="n"/>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="A20" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Taskbar animation cache cleanup</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Clean up stale animation/taskbar caches and completed animation cancellation tokens.</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Appearance apply now prunes handles no longer present in the live taskbar set and clears completed animation cancellation state without waiting for the next animation.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n"/>
@@ -3981,11 +4007,20 @@
       <c r="F29" s="11" t="n"/>
       <c r="G29" s="11" t="n"/>
     </row>
+    <row r="30">
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F29">
+  <conditionalFormatting sqref="F5:F30">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -3999,7 +4034,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E29">
+  <conditionalFormatting sqref="E5:E30">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4014,10 +4049,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Guard no-op AppState setters
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-73</t>
+74</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-73</t>
+74</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3927,13 +3927,39 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="n"/>
-      <c r="B21" s="11" t="n"/>
-      <c r="C21" s="11" t="n"/>
-      <c r="D21" s="11" t="n"/>
-      <c r="E21" s="11" t="n"/>
-      <c r="F21" s="11" t="n"/>
-      <c r="G21" s="11" t="n"/>
+      <c r="A21" s="8" t="n">
+        <v>74</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>AppState no-op setter guards</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>Avoid redundant save, notify, apply, tray, startup, and hotkey work when requested settings already match current state.</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>State setters now short-circuit duplicate values while preserving debounced preview commits and retry paths for failed startup or hotkey registration.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n"/>
@@ -4016,11 +4042,20 @@
       <c r="F30" s="10" t="n"/>
       <c r="G30" s="10" t="n"/>
     </row>
+    <row r="31">
+      <c r="A31" s="11" t="n"/>
+      <c r="B31" s="11" t="n"/>
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="11" t="n"/>
+      <c r="E31" s="11" t="n"/>
+      <c r="F31" s="11" t="n"/>
+      <c r="G31" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F30">
+  <conditionalFormatting sqref="F5:F31">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4034,7 +4069,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E30">
+  <conditionalFormatting sqref="E5:E31">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4049,10 +4084,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Skip redundant page navigation
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-74</t>
+75</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-74</t>
+75</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3962,13 +3962,39 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="n"/>
-      <c r="B22" s="10" t="n"/>
-      <c r="C22" s="10" t="n"/>
-      <c r="D22" s="10" t="n"/>
-      <c r="E22" s="10" t="n"/>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
+      <c r="A22" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Same-page navigation no-op guard</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Avoid recreating the current WinUI page when tray, hotkey, or navigation requests target the page already displayed.</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>Main window navigation now skips same-page requests so loaded pages keep their existing controls, timers, and subscriptions instead of churning through unload/reload work.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n"/>
@@ -4051,11 +4077,20 @@
       <c r="F31" s="11" t="n"/>
       <c r="G31" s="11" t="n"/>
     </row>
+    <row r="32">
+      <c r="A32" s="10" t="n"/>
+      <c r="B32" s="10" t="n"/>
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="10" t="n"/>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="10" t="n"/>
+      <c r="G32" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F31">
+  <conditionalFormatting sqref="F5:F32">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4069,7 +4104,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E31">
+  <conditionalFormatting sqref="E5:E32">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4084,10 +4119,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Optimize runtime history refresh checks
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-75</t>
+76</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-75</t>
+76</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3997,13 +3997,39 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="n"/>
-      <c r="B23" s="11" t="n"/>
-      <c r="C23" s="11" t="n"/>
-      <c r="D23" s="11" t="n"/>
-      <c r="E23" s="11" t="n"/>
-      <c r="F23" s="11" t="n"/>
-      <c r="G23" s="11" t="n"/>
+      <c r="A23" s="8" t="n">
+        <v>76</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Runtime event refresh versioning</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>Avoid rebuilding runtime history signature strings on every Dashboard, Monitors, and Diagnostics refresh.</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>RuntimeSnapshot now exposes a RecentEventsVersion counter so pages use integer change checks before rebuilding history list item sources.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n"/>
@@ -4086,11 +4112,20 @@
       <c r="F32" s="10" t="n"/>
       <c r="G32" s="10" t="n"/>
     </row>
+    <row r="33">
+      <c r="A33" s="11" t="n"/>
+      <c r="B33" s="11" t="n"/>
+      <c r="C33" s="11" t="n"/>
+      <c r="D33" s="11" t="n"/>
+      <c r="E33" s="11" t="n"/>
+      <c r="F33" s="11" t="n"/>
+      <c r="G33" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F32">
+  <conditionalFormatting sqref="F5:F33">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4104,7 +4139,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E32">
+  <conditionalFormatting sqref="E5:E33">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4119,10 +4154,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Optimize monitor overview refresh checks
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-76</t>
+77</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-76</t>
+77</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4032,13 +4032,39 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="n"/>
-      <c r="B24" s="10" t="n"/>
-      <c r="C24" s="10" t="n"/>
-      <c r="D24" s="10" t="n"/>
-      <c r="E24" s="10" t="n"/>
-      <c r="F24" s="10" t="n"/>
-      <c r="G24" s="10" t="n"/>
+      <c r="A24" s="9" t="n">
+        <v>77</v>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Monitor list refresh versioning</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Avoid rebuilding monitor overview signature strings on every Monitors page refresh.</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>AppState now tracks MonitorsVersion so monitor overview rows rebuild only when the live monitor collection or overrides change.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="n"/>
@@ -4121,11 +4147,20 @@
       <c r="F33" s="11" t="n"/>
       <c r="G33" s="11" t="n"/>
     </row>
+    <row r="34">
+      <c r="A34" s="10" t="n"/>
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="10" t="n"/>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="10" t="n"/>
+      <c r="G34" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F33">
+  <conditionalFormatting sqref="F5:F34">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4139,7 +4174,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E33">
+  <conditionalFormatting sqref="E5:E34">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4154,10 +4189,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Coalesce loaded page refreshes
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-77</t>
+78</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-77</t>
+78</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4067,13 +4067,39 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="n"/>
-      <c r="B25" s="11" t="n"/>
-      <c r="C25" s="11" t="n"/>
-      <c r="D25" s="11" t="n"/>
-      <c r="E25" s="11" t="n"/>
-      <c r="F25" s="11" t="n"/>
-      <c r="G25" s="11" t="n"/>
+      <c r="A25" s="8" t="n">
+        <v>78</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Loaded page refresh coalescing</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Avoid queuing duplicate UI refreshes for loaded pages during quick AppState change bursts.</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>State-listening pages now share a RefreshCoalescer so repeated change notifications collapse to one pending dispatcher refresh per page.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n"/>
@@ -4156,11 +4182,20 @@
       <c r="F34" s="10" t="n"/>
       <c r="G34" s="10" t="n"/>
     </row>
+    <row r="35">
+      <c r="A35" s="11" t="n"/>
+      <c r="B35" s="11" t="n"/>
+      <c r="C35" s="11" t="n"/>
+      <c r="D35" s="11" t="n"/>
+      <c r="E35" s="11" t="n"/>
+      <c r="F35" s="11" t="n"/>
+      <c r="G35" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F34">
+  <conditionalFormatting sqref="F5:F35">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4174,7 +4209,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E34">
+  <conditionalFormatting sqref="E5:E35">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4189,10 +4224,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Skip synced monitor apply lookup
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-78</t>
+79</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-78</t>
+79</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4102,13 +4102,39 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="n"/>
-      <c r="B26" s="10" t="n"/>
-      <c r="C26" s="10" t="n"/>
-      <c r="D26" s="10" t="n"/>
-      <c r="E26" s="10" t="n"/>
-      <c r="F26" s="10" t="n"/>
-      <c r="G26" s="10" t="n"/>
+      <c r="A26" s="9" t="n">
+        <v>79</v>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Synced monitor apply lookup skip</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Avoid building per-monitor override lookup dictionaries when all monitors follow the primary opacity.</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>TaskbarAppearanceService now creates the monitor override lookup only when at least one monitor is unsynced.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n"/>
@@ -4191,11 +4217,20 @@
       <c r="F35" s="11" t="n"/>
       <c r="G35" s="11" t="n"/>
     </row>
+    <row r="36">
+      <c r="A36" s="10" t="n"/>
+      <c r="B36" s="10" t="n"/>
+      <c r="C36" s="10" t="n"/>
+      <c r="D36" s="10" t="n"/>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F35">
+  <conditionalFormatting sqref="F5:F36">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4209,7 +4244,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E35">
+  <conditionalFormatting sqref="E5:E36">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4224,10 +4259,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add taskbar apply diagnostics counters
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-79</t>
+80</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-79</t>
+80</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4137,13 +4137,39 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="n"/>
-      <c r="B27" s="11" t="n"/>
-      <c r="C27" s="11" t="n"/>
-      <c r="D27" s="11" t="n"/>
-      <c r="E27" s="11" t="n"/>
-      <c r="F27" s="11" t="n"/>
-      <c r="G27" s="11" t="n"/>
+      <c r="A27" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Taskbar apply diagnostics counters</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>Expose lightweight counters for native composition skips, alpha skips, monitor lookup use, and animation starts.</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>Diagnostics now shows latest apply counters so future optimization passes can be guided by measured skip behavior instead of source inspection alone.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n"/>
@@ -4226,11 +4252,20 @@
       <c r="F36" s="10" t="n"/>
       <c r="G36" s="10" t="n"/>
     </row>
+    <row r="37">
+      <c r="A37" s="11" t="n"/>
+      <c r="B37" s="11" t="n"/>
+      <c r="C37" s="11" t="n"/>
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="11" t="n"/>
+      <c r="G37" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F36">
+  <conditionalFormatting sqref="F5:F37">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4244,7 +4279,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E36">
+  <conditionalFormatting sqref="E5:E37">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4259,10 +4294,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reduce layered alpha apply allocations
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-80</t>
+81</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-80</t>
+81</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4172,13 +4172,39 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="n"/>
-      <c r="B28" s="10" t="n"/>
-      <c r="C28" s="10" t="n"/>
-      <c r="D28" s="10" t="n"/>
-      <c r="E28" s="10" t="n"/>
-      <c r="F28" s="10" t="n"/>
-      <c r="G28" s="10" t="n"/>
+      <c r="A28" s="9" t="n">
+        <v>81</v>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Layered alpha change loop allocation reduction</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Avoid LINQ iterator and dictionary projection overhead while collecting changed layered-alpha targets.</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>TaskbarAppearanceService now builds alpha-change targets in one pre-sized loop while preserving skip counters for Diagnostics.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="n"/>
@@ -4261,11 +4287,20 @@
       <c r="F37" s="11" t="n"/>
       <c r="G37" s="11" t="n"/>
     </row>
+    <row r="38">
+      <c r="A38" s="10" t="n"/>
+      <c r="B38" s="10" t="n"/>
+      <c r="C38" s="10" t="n"/>
+      <c r="D38" s="10" t="n"/>
+      <c r="E38" s="10" t="n"/>
+      <c r="F38" s="10" t="n"/>
+      <c r="G38" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F37">
+  <conditionalFormatting sqref="F5:F38">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4279,7 +4314,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E37">
+  <conditionalFormatting sqref="E5:E38">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4294,10 +4329,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E37" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reduce taskbar target dedupe allocations
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-81</t>
+82</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-81</t>
+82</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4207,13 +4207,39 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="n"/>
-      <c r="B29" s="11" t="n"/>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="11" t="n"/>
-      <c r="E29" s="11" t="n"/>
-      <c r="F29" s="11" t="n"/>
-      <c r="G29" s="11" t="n"/>
+      <c r="A29" s="8" t="n">
+        <v>82</v>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Taskbar target dedupe allocation reduction</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Avoid LINQ grouping when de-duplicating taskbar targets by window handle before apply.</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>TaskbarAppearanceService now preserves first target per handle with a single loop and pre-sizes per-apply target dictionaries.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n"/>
@@ -4296,11 +4322,20 @@
       <c r="F38" s="10" t="n"/>
       <c r="G38" s="10" t="n"/>
     </row>
+    <row r="39">
+      <c r="A39" s="11" t="n"/>
+      <c r="B39" s="11" t="n"/>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="11" t="n"/>
+      <c r="G39" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F38">
+  <conditionalFormatting sqref="F5:F39">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4314,7 +4349,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E38">
+  <conditionalFormatting sqref="E5:E39">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4329,10 +4364,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reduce stale taskbar cache pruning allocations
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-82</t>
+83</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-82</t>
+83</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4242,13 +4242,39 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="n"/>
-      <c r="B30" s="10" t="n"/>
-      <c r="C30" s="10" t="n"/>
-      <c r="D30" s="10" t="n"/>
-      <c r="E30" s="10" t="n"/>
-      <c r="F30" s="10" t="n"/>
-      <c r="G30" s="10" t="n"/>
+      <c r="A30" s="9" t="n">
+        <v>83</v>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Stale taskbar cache pruning allocation reduction</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Avoid LINQ projection and stale-handle arrays while pruning cached taskbar state after apply.</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>TaskbarAppearanceService now prunes alpha and appearance caches directly against one live handle set built from current taskbar targets.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n"/>
@@ -4331,11 +4357,20 @@
       <c r="F39" s="11" t="n"/>
       <c r="G39" s="11" t="n"/>
     </row>
+    <row r="40">
+      <c r="A40" s="10" t="n"/>
+      <c r="B40" s="10" t="n"/>
+      <c r="C40" s="10" t="n"/>
+      <c r="D40" s="10" t="n"/>
+      <c r="E40" s="10" t="n"/>
+      <c r="F40" s="10" t="n"/>
+      <c r="G40" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F39">
+  <conditionalFormatting sqref="F5:F40">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4349,7 +4384,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E39">
+  <conditionalFormatting sqref="E5:E40">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4364,10 +4399,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reduce monitor override lookup allocations
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-83</t>
+84</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-83</t>
+84</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4277,13 +4277,39 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="n"/>
-      <c r="B31" s="11" t="n"/>
-      <c r="C31" s="11" t="n"/>
-      <c r="D31" s="11" t="n"/>
-      <c r="E31" s="11" t="n"/>
-      <c r="F31" s="11" t="n"/>
-      <c r="G31" s="11" t="n"/>
+      <c r="A31" s="8" t="n">
+        <v>84</v>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Monitor override lookup loop allocation reduction</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>Avoid double-scanning and LINQ grouping when building per-monitor override lookup data.</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F31" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
+          <t>TaskbarAppearanceService now builds unsynced monitor override lookup entries in one loop and returns no dictionary for fully synced monitor sets.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n"/>
@@ -4366,11 +4392,20 @@
       <c r="F40" s="10" t="n"/>
       <c r="G40" s="10" t="n"/>
     </row>
+    <row r="41">
+      <c r="A41" s="11" t="n"/>
+      <c r="B41" s="11" t="n"/>
+      <c r="C41" s="11" t="n"/>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="11" t="n"/>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F40">
+  <conditionalFormatting sqref="F5:F41">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4384,7 +4419,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E40">
+  <conditionalFormatting sqref="E5:E41">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4399,10 +4434,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reduce taskbar catalog enumeration allocations
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-84</t>
+85</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-84</t>
+85</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4312,13 +4312,39 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="n"/>
-      <c r="B32" s="10" t="n"/>
-      <c r="C32" s="10" t="n"/>
-      <c r="D32" s="10" t="n"/>
-      <c r="E32" s="10" t="n"/>
-      <c r="F32" s="10" t="n"/>
-      <c r="G32" s="10" t="n"/>
+      <c r="A32" s="9" t="n">
+        <v>85</v>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Taskbar catalog iterator allocation reduction</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>Avoid iterator and array materialization when collecting current taskbar windows.</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>TaskbarWindowCatalog now builds the current taskbar list directly with a small pre-sized list instead of yielding and materializing an array.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="n"/>
@@ -4401,11 +4427,20 @@
       <c r="F41" s="11" t="n"/>
       <c r="G41" s="11" t="n"/>
     </row>
+    <row r="42">
+      <c r="A42" s="10" t="n"/>
+      <c r="B42" s="10" t="n"/>
+      <c r="C42" s="10" t="n"/>
+      <c r="D42" s="10" t="n"/>
+      <c r="E42" s="10" t="n"/>
+      <c r="F42" s="10" t="n"/>
+      <c r="G42" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F41">
+  <conditionalFormatting sqref="F5:F42">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4419,7 +4454,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E41">
+  <conditionalFormatting sqref="E5:E42">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4434,10 +4469,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reduce fade duration projection allocations
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-85</t>
+86</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-85</t>
+86</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4347,13 +4347,39 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="n"/>
-      <c r="B33" s="11" t="n"/>
-      <c r="C33" s="11" t="n"/>
-      <c r="D33" s="11" t="n"/>
-      <c r="E33" s="11" t="n"/>
-      <c r="F33" s="11" t="n"/>
-      <c r="G33" s="11" t="n"/>
+      <c r="A33" s="8" t="n">
+        <v>86</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Fade duration projection allocation reduction</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Avoid LINQ dictionary projections and duration scans when preparing taskbar fade animations.</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>TaskbarAppearanceService now builds animation start and duration dictionaries with pre-sized loops and checks for animated durations with a direct scan.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n"/>
@@ -4436,11 +4462,20 @@
       <c r="F42" s="10" t="n"/>
       <c r="G42" s="10" t="n"/>
     </row>
+    <row r="43">
+      <c r="A43" s="11" t="n"/>
+      <c r="B43" s="11" t="n"/>
+      <c r="C43" s="11" t="n"/>
+      <c r="D43" s="11" t="n"/>
+      <c r="E43" s="11" t="n"/>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F42">
+  <conditionalFormatting sqref="F5:F43">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4454,7 +4489,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E42">
+  <conditionalFormatting sqref="E5:E43">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4469,10 +4504,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Optimize monitor sequence comparisons
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-86</t>
+87</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-86</t>
+87</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4382,13 +4382,39 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="n"/>
-      <c r="B34" s="10" t="n"/>
-      <c r="C34" s="10" t="n"/>
-      <c r="D34" s="10" t="n"/>
-      <c r="E34" s="10" t="n"/>
-      <c r="F34" s="10" t="n"/>
-      <c r="G34" s="10" t="n"/>
+      <c r="A34" s="9" t="n">
+        <v>87</v>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Monitor sequence comparison fast path</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>Avoid enumerator churn when comparing list-backed monitor profiles during refresh.</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>MonitorProfile.SequenceMatches now compares IList-backed monitor collections by count and index while preserving the deferred enumerable fallback.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="n"/>
@@ -4471,11 +4497,20 @@
       <c r="F43" s="11" t="n"/>
       <c r="G43" s="11" t="n"/>
     </row>
+    <row r="44">
+      <c r="A44" s="10" t="n"/>
+      <c r="B44" s="10" t="n"/>
+      <c r="C44" s="10" t="n"/>
+      <c r="D44" s="10" t="n"/>
+      <c r="E44" s="10" t="n"/>
+      <c r="F44" s="10" t="n"/>
+      <c r="G44" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F43">
+  <conditionalFormatting sqref="F5:F44">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4489,7 +4524,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E43">
+  <conditionalFormatting sqref="E5:E44">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4504,10 +4539,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Optimize monitor refresh merging
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-87</t>
+88</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-87</t>
+88</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4417,13 +4417,39 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="n"/>
-      <c r="B35" s="11" t="n"/>
-      <c r="C35" s="11" t="n"/>
-      <c r="D35" s="11" t="n"/>
-      <c r="E35" s="11" t="n"/>
-      <c r="F35" s="11" t="n"/>
-      <c r="G35" s="11" t="n"/>
+      <c r="A35" s="8" t="n">
+        <v>88</v>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Monitor refresh merge loop optimization</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>Avoid LINQ projection and delegate searches when merging detected monitor data with saved overrides.</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>AppState.RefreshMonitors now uses a pre-sized MonitorProfile merge helper with direct device-name lookup loops while preserving saved per-monitor overrides.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n"/>
@@ -4506,11 +4532,20 @@
       <c r="F44" s="10" t="n"/>
       <c r="G44" s="10" t="n"/>
     </row>
+    <row r="45">
+      <c r="A45" s="11" t="n"/>
+      <c r="B45" s="11" t="n"/>
+      <c r="C45" s="11" t="n"/>
+      <c r="D45" s="11" t="n"/>
+      <c r="E45" s="11" t="n"/>
+      <c r="F45" s="11" t="n"/>
+      <c r="G45" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F44">
+  <conditionalFormatting sqref="F5:F45">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4524,7 +4559,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E44">
+  <conditionalFormatting sqref="E5:E45">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4539,10 +4574,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reduce monitor catalog ordering allocations
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-88</t>
+89</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-88</t>
+89</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4452,13 +4452,39 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="n"/>
-      <c r="B36" s="10" t="n"/>
-      <c r="C36" s="10" t="n"/>
-      <c r="D36" s="10" t="n"/>
-      <c r="E36" s="10" t="n"/>
-      <c r="F36" s="10" t="n"/>
-      <c r="G36" s="10" t="n"/>
+      <c r="A36" s="9" t="n">
+        <v>89</v>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Monitor catalog ordering allocation reduction</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Avoid LINQ ordering and array materialization when building detected monitor profiles.</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>MonitorCatalog now builds a pre-sized profile list directly, keeps primary displays first during insertion, and preserves discovery-based display names.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n"/>
@@ -4541,11 +4567,20 @@
       <c r="F45" s="11" t="n"/>
       <c r="G45" s="11" t="n"/>
     </row>
+    <row r="46">
+      <c r="A46" s="10" t="n"/>
+      <c r="B46" s="10" t="n"/>
+      <c r="C46" s="10" t="n"/>
+      <c r="D46" s="10" t="n"/>
+      <c r="E46" s="10" t="n"/>
+      <c r="F46" s="10" t="n"/>
+      <c r="G46" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F45">
+  <conditionalFormatting sqref="F5:F46">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4559,7 +4594,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E45">
+  <conditionalFormatting sqref="E5:E46">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4574,10 +4609,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Optimize monitor override lookups
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-89</t>
+90</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-89</t>
+90</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4487,13 +4487,39 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="11" t="n"/>
-      <c r="B37" s="11" t="n"/>
-      <c r="C37" s="11" t="n"/>
-      <c r="D37" s="11" t="n"/>
-      <c r="E37" s="11" t="n"/>
-      <c r="F37" s="11" t="n"/>
-      <c r="G37" s="11" t="n"/>
+      <c r="A37" s="8" t="n">
+        <v>90</v>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Monitor override lookup fast path</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>Avoid delegate-based FirstOrDefault searches when applying per-monitor overrides.</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>AppState.SetMonitorOverride now reuses a list-aware MonitorProfile device lookup helper for saved and live monitor updates while preserving case-insensitive matching.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n"/>
@@ -4576,11 +4602,20 @@
       <c r="F46" s="10" t="n"/>
       <c r="G46" s="10" t="n"/>
     </row>
+    <row r="47">
+      <c r="A47" s="11" t="n"/>
+      <c r="B47" s="11" t="n"/>
+      <c r="C47" s="11" t="n"/>
+      <c r="D47" s="11" t="n"/>
+      <c r="E47" s="11" t="n"/>
+      <c r="F47" s="11" t="n"/>
+      <c r="G47" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F46">
+  <conditionalFormatting sqref="F5:F47">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4594,7 +4629,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E46">
+  <conditionalFormatting sqref="E5:E47">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4609,10 +4644,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Optimize monitor page refresh scans
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-90</t>
+91</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-90</t>
+91</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4522,13 +4522,39 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="n"/>
-      <c r="B38" s="10" t="n"/>
-      <c r="C38" s="10" t="n"/>
-      <c r="D38" s="10" t="n"/>
-      <c r="E38" s="10" t="n"/>
-      <c r="F38" s="10" t="n"/>
-      <c r="G38" s="10" t="n"/>
+      <c r="A38" s="9" t="n">
+        <v>91</v>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Monitor page refresh scan fast paths</t>
+        </is>
+      </c>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>Avoid delegate-based monitor count and selected-display scans during Monitors page refresh.</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>Monitors page now uses list-aware MonitorProfile helpers for synced display counts and secondary-or-primary selection.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="n"/>
@@ -4611,11 +4637,20 @@
       <c r="F47" s="11" t="n"/>
       <c r="G47" s="11" t="n"/>
     </row>
+    <row r="48">
+      <c r="A48" s="10" t="n"/>
+      <c r="B48" s="10" t="n"/>
+      <c r="C48" s="10" t="n"/>
+      <c r="D48" s="10" t="n"/>
+      <c r="E48" s="10" t="n"/>
+      <c r="F48" s="10" t="n"/>
+      <c r="G48" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F47">
+  <conditionalFormatting sqref="F5:F48">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4629,7 +4664,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E47">
+  <conditionalFormatting sqref="E5:E48">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4644,10 +4679,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reduce runtime event list projection allocations
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-91</t>
+92</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-91</t>
+92</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4557,13 +4557,39 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="n"/>
-      <c r="B39" s="11" t="n"/>
-      <c r="C39" s="11" t="n"/>
-      <c r="D39" s="11" t="n"/>
-      <c r="E39" s="11" t="n"/>
-      <c r="F39" s="11" t="n"/>
-      <c r="G39" s="11" t="n"/>
+      <c r="A39" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Runtime event list projection allocation reduction</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>Avoid LINQ projection allocations when rebuilding version-gated runtime event lists.</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Dashboard, Diagnostics, and Monitors now rebuild runtime event list rows with pre-sized loops while preserving existing row text.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n"/>
@@ -4646,11 +4672,20 @@
       <c r="F48" s="10" t="n"/>
       <c r="G48" s="10" t="n"/>
     </row>
+    <row r="49">
+      <c r="A49" s="11" t="n"/>
+      <c r="B49" s="11" t="n"/>
+      <c r="C49" s="11" t="n"/>
+      <c r="D49" s="11" t="n"/>
+      <c r="E49" s="11" t="n"/>
+      <c r="F49" s="11" t="n"/>
+      <c r="G49" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F48">
+  <conditionalFormatting sqref="F5:F49">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4664,7 +4699,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E48">
+  <conditionalFormatting sqref="E5:E49">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4679,10 +4714,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Pre-size taskbar handle sets
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-92</t>
+93</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-92</t>
+93</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4592,13 +4592,39 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="n"/>
-      <c r="B40" s="10" t="n"/>
-      <c r="C40" s="10" t="n"/>
-      <c r="D40" s="10" t="n"/>
-      <c r="E40" s="10" t="n"/>
-      <c r="F40" s="10" t="n"/>
-      <c r="G40" s="10" t="n"/>
+      <c r="A40" s="9" t="n">
+        <v>93</v>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Taskbar apply handle set pre-sizing</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>Avoid avoidable HashSet growth while deduplicating and pruning taskbar handles during apply.</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G40" s="9" t="inlineStr">
+        <is>
+          <t>TaskbarAppearanceService now pre-sizes handle sets from known target counts in DistinctByHandle and live-cache pruning.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="11" t="n"/>
@@ -4681,11 +4707,20 @@
       <c r="F49" s="11" t="n"/>
       <c r="G49" s="11" t="n"/>
     </row>
+    <row r="50">
+      <c r="A50" s="10" t="n"/>
+      <c r="B50" s="10" t="n"/>
+      <c r="C50" s="10" t="n"/>
+      <c r="D50" s="10" t="n"/>
+      <c r="E50" s="10" t="n"/>
+      <c r="F50" s="10" t="n"/>
+      <c r="G50" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F49">
+  <conditionalFormatting sqref="F5:F50">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4699,7 +4734,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E49">
+  <conditionalFormatting sqref="E5:E50">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4714,10 +4749,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E49" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Gate runtime sensor native checks
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-93</t>
+94</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-93</t>
+94</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4627,13 +4627,39 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="n"/>
-      <c r="B41" s="11" t="n"/>
-      <c r="C41" s="11" t="n"/>
-      <c r="D41" s="11" t="n"/>
-      <c r="E41" s="11" t="n"/>
-      <c r="F41" s="11" t="n"/>
-      <c r="G41" s="11" t="n"/>
+      <c r="A41" s="8" t="n">
+        <v>94</v>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Runtime sensor native check gating</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Skip unneeded native foreground, fullscreen, and taskbar proximity checks based on automation settings.</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t>RuntimeStateSensorService now returns Desktop immediately when automation is disabled and only runs fullscreen or hover/taskbar checks when those policies are enabled.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n"/>
@@ -4716,11 +4742,20 @@
       <c r="F50" s="10" t="n"/>
       <c r="G50" s="10" t="n"/>
     </row>
+    <row r="51">
+      <c r="A51" s="11" t="n"/>
+      <c r="B51" s="11" t="n"/>
+      <c r="C51" s="11" t="n"/>
+      <c r="D51" s="11" t="n"/>
+      <c r="E51" s="11" t="n"/>
+      <c r="F51" s="11" t="n"/>
+      <c r="G51" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F50">
+  <conditionalFormatting sqref="F5:F51">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4734,7 +4769,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E50">
+  <conditionalFormatting sqref="E5:E51">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4749,10 +4784,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Short-circuit runtime hover sensing
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-94</t>
+95</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-94</t>
+95</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4662,13 +4662,39 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="10" t="n"/>
-      <c r="B42" s="10" t="n"/>
-      <c r="C42" s="10" t="n"/>
-      <c r="D42" s="10" t="n"/>
-      <c r="E42" s="10" t="n"/>
-      <c r="F42" s="10" t="n"/>
-      <c r="G42" s="10" t="n"/>
+      <c r="A42" s="9" t="n">
+        <v>95</v>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Runtime sensor hover priority short-circuit</t>
+        </is>
+      </c>
+      <c r="D42" s="9" t="inlineStr">
+        <is>
+          <t>Skip foreground, maximize, and fullscreen native checks when hover proximity already resolves the active runtime trigger.</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>RuntimeStateSensorService now checks hover proximity first after automation gating and returns Hover immediately when active.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="n"/>
@@ -4751,11 +4777,20 @@
       <c r="F51" s="11" t="n"/>
       <c r="G51" s="11" t="n"/>
     </row>
+    <row r="52">
+      <c r="A52" s="10" t="n"/>
+      <c r="B52" s="10" t="n"/>
+      <c r="C52" s="10" t="n"/>
+      <c r="D52" s="10" t="n"/>
+      <c r="E52" s="10" t="n"/>
+      <c r="F52" s="10" t="n"/>
+      <c r="G52" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F51">
+  <conditionalFormatting sqref="F5:F52">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4769,7 +4804,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E51">
+  <conditionalFormatting sqref="E5:E52">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4784,10 +4819,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reuse runtime sensor class-name buffer
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-95</t>
+96</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-95</t>
+96</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4697,13 +4697,39 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="n"/>
-      <c r="B43" s="11" t="n"/>
-      <c r="C43" s="11" t="n"/>
-      <c r="D43" s="11" t="n"/>
-      <c r="E43" s="11" t="n"/>
-      <c r="F43" s="11" t="n"/>
-      <c r="G43" s="11" t="n"/>
+      <c r="A43" s="8" t="n">
+        <v>96</v>
+      </c>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Runtime sensor shell class buffer reuse</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="inlineStr">
+        <is>
+          <t>Avoid allocating a new class-name StringBuilder during each foreground shell-window check.</t>
+        </is>
+      </c>
+      <c r="E43" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F43" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t>RuntimeStateSensorService now reuses one class-name buffer per sensor instance and keeps shell class matching covered by tests.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n"/>
@@ -4786,11 +4812,20 @@
       <c r="F52" s="10" t="n"/>
       <c r="G52" s="10" t="n"/>
     </row>
+    <row r="53">
+      <c r="A53" s="11" t="n"/>
+      <c r="B53" s="11" t="n"/>
+      <c r="C53" s="11" t="n"/>
+      <c r="D53" s="11" t="n"/>
+      <c r="E53" s="11" t="n"/>
+      <c r="F53" s="11" t="n"/>
+      <c r="G53" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F52">
+  <conditionalFormatting sqref="F5:F53">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4804,7 +4839,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E52">
+  <conditionalFormatting sqref="E5:E53">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4819,10 +4854,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Cache unchanged settings saves
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-96</t>
+97</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-96</t>
+97</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4732,13 +4732,39 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="10" t="n"/>
-      <c r="B44" s="10" t="n"/>
-      <c r="C44" s="10" t="n"/>
-      <c r="D44" s="10" t="n"/>
-      <c r="E44" s="10" t="n"/>
-      <c r="F44" s="10" t="n"/>
-      <c r="G44" s="10" t="n"/>
+      <c r="A44" s="9" t="n">
+        <v>97</v>
+      </c>
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="inlineStr">
+        <is>
+          <t>Settings save cache</t>
+        </is>
+      </c>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>Avoid reading settings.json during ordinary unchanged in-process saves.</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G44" s="9" t="inlineStr">
+        <is>
+          <t>SettingsStore now caches the last serialized settings and file timestamp so unchanged saves can skip disk reads while still detecting external file edits.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="n"/>
@@ -4821,11 +4847,20 @@
       <c r="F53" s="11" t="n"/>
       <c r="G53" s="11" t="n"/>
     </row>
+    <row r="54">
+      <c r="A54" s="10" t="n"/>
+      <c r="B54" s="10" t="n"/>
+      <c r="C54" s="10" t="n"/>
+      <c r="D54" s="10" t="n"/>
+      <c r="E54" s="10" t="n"/>
+      <c r="F54" s="10" t="n"/>
+      <c r="G54" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F53">
+  <conditionalFormatting sqref="F5:F54">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4839,7 +4874,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E53">
+  <conditionalFormatting sqref="E5:E54">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4854,10 +4889,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Reuse startup taskbar catalog
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-97</t>
+98</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-97</t>
+98</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4767,13 +4767,39 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="11" t="n"/>
-      <c r="B45" s="11" t="n"/>
-      <c r="C45" s="11" t="n"/>
-      <c r="D45" s="11" t="n"/>
-      <c r="E45" s="11" t="n"/>
-      <c r="F45" s="11" t="n"/>
-      <c r="G45" s="11" t="n"/>
+      <c r="A45" s="8" t="n">
+        <v>98</v>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Startup taskbar catalog reuse</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="inlineStr">
+        <is>
+          <t>Avoid enumerating taskbar windows twice during launch initialization.</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G45" s="8" t="inlineStr">
+        <is>
+          <t>AppState now captures the startup taskbar snapshot once, uses it for monitor profile refresh, and reuses it for the initial taskbar apply while later applies still refresh live targets.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n"/>
@@ -4856,11 +4882,20 @@
       <c r="F54" s="10" t="n"/>
       <c r="G54" s="10" t="n"/>
     </row>
+    <row r="55">
+      <c r="A55" s="11" t="n"/>
+      <c r="B55" s="11" t="n"/>
+      <c r="C55" s="11" t="n"/>
+      <c r="D55" s="11" t="n"/>
+      <c r="E55" s="11" t="n"/>
+      <c r="F55" s="11" t="n"/>
+      <c r="G55" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F54">
+  <conditionalFormatting sqref="F5:F55">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4874,7 +4909,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E54">
+  <conditionalFormatting sqref="E5:E55">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4889,10 +4924,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Precompute fade animation tracks
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-98</t>
+99</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-98</t>
+99</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4802,13 +4802,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="10" t="n"/>
-      <c r="B46" s="10" t="n"/>
-      <c r="C46" s="10" t="n"/>
-      <c r="D46" s="10" t="n"/>
-      <c r="E46" s="10" t="n"/>
-      <c r="F46" s="10" t="n"/>
-      <c r="G46" s="10" t="n"/>
+      <c r="A46" s="9" t="n">
+        <v>99</v>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="inlineStr">
+        <is>
+          <t>Fade animation track precompute</t>
+        </is>
+      </c>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>Reduce dictionary lookups during each taskbar fade animation frame.</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>TaskbarAppearanceService now precomputes alpha animation tracks once per fade so the frame loop iterates direct handle/start/target/duration values.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="11" t="n"/>
@@ -4891,11 +4917,20 @@
       <c r="F55" s="11" t="n"/>
       <c r="G55" s="11" t="n"/>
     </row>
+    <row r="56">
+      <c r="A56" s="10" t="n"/>
+      <c r="B56" s="10" t="n"/>
+      <c r="C56" s="10" t="n"/>
+      <c r="D56" s="10" t="n"/>
+      <c r="E56" s="10" t="n"/>
+      <c r="F56" s="10" t="n"/>
+      <c r="G56" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F55">
+  <conditionalFormatting sqref="F5:F56">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4909,7 +4944,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E55">
+  <conditionalFormatting sqref="E5:E56">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4924,10 +4959,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Cache layered taskbar style checks
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-99</t>
+100</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-99</t>
+100</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4837,13 +4837,39 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="11" t="n"/>
-      <c r="B47" s="11" t="n"/>
-      <c r="C47" s="11" t="n"/>
-      <c r="D47" s="11" t="n"/>
-      <c r="E47" s="11" t="n"/>
-      <c r="F47" s="11" t="n"/>
-      <c r="G47" s="11" t="n"/>
+      <c r="A47" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Layered style check cache</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="inlineStr">
+        <is>
+          <t>Avoid repeated native style reads for taskbar handles already known to be layered.</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
+          <t>TaskbarAppearanceService now caches handles after layered style verification or setup and prunes that cache with stale taskbar handles.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n"/>
@@ -4926,11 +4952,20 @@
       <c r="F56" s="10" t="n"/>
       <c r="G56" s="10" t="n"/>
     </row>
+    <row r="57">
+      <c r="A57" s="11" t="n"/>
+      <c r="B57" s="11" t="n"/>
+      <c r="C57" s="11" t="n"/>
+      <c r="D57" s="11" t="n"/>
+      <c r="E57" s="11" t="n"/>
+      <c r="F57" s="11" t="n"/>
+      <c r="G57" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F56">
+  <conditionalFormatting sqref="F5:F57">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4944,7 +4979,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E56">
+  <conditionalFormatting sqref="E5:E57">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4959,10 +4994,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Optimize taskbar cache pruning
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-100</t>
+101</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-100</t>
+101</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4872,13 +4872,39 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="10" t="n"/>
-      <c r="B48" s="10" t="n"/>
-      <c r="C48" s="10" t="n"/>
-      <c r="D48" s="10" t="n"/>
-      <c r="E48" s="10" t="n"/>
-      <c r="F48" s="10" t="n"/>
-      <c r="G48" s="10" t="n"/>
+      <c r="A48" s="9" t="n">
+        <v>101</v>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Concurrent cache prune enumeration</t>
+        </is>
+      </c>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>Avoid separate key-collection enumeration while pruning stale taskbar apply caches.</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>TaskbarAppearanceService now enumerates concurrent cache entries directly when pruning alpha, appearance, and layered-style caches after each apply.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="n"/>
@@ -4961,11 +4987,20 @@
       <c r="F57" s="11" t="n"/>
       <c r="G57" s="11" t="n"/>
     </row>
+    <row r="58">
+      <c r="A58" s="10" t="n"/>
+      <c r="B58" s="10" t="n"/>
+      <c r="C58" s="10" t="n"/>
+      <c r="D58" s="10" t="n"/>
+      <c r="E58" s="10" t="n"/>
+      <c r="F58" s="10" t="n"/>
+      <c r="G58" s="10" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F57">
+  <conditionalFormatting sqref="F5:F58">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -4979,7 +5014,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E57">
+  <conditionalFormatting sqref="E5:E58">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -4994,10 +5029,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add final production optimization audit
</commit_message>
<xml_diff>
--- a/tracker/Project-Tracker.xlsx
+++ b/tracker/Project-Tracker.xlsx
@@ -614,13 +614,13 @@
       <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Total
-101</t>
+102</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Done
-101</t>
+102</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -3309,7 +3309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4907,13 +4907,39 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="11" t="n"/>
-      <c r="B49" s="11" t="n"/>
-      <c r="C49" s="11" t="n"/>
-      <c r="D49" s="11" t="n"/>
-      <c r="E49" s="11" t="n"/>
-      <c r="F49" s="11" t="n"/>
-      <c r="G49" s="11" t="n"/>
+      <c r="A49" s="8" t="n">
+        <v>102</v>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Final production allocation audit</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Classify remaining production allocation and native-work search hits after the optimization suite.</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>Final audit report records remaining hits as necessary settings I/O, pre-sized runtime collections, UI-binding rows, or test-only helpers with no further code change justified by current evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="10" t="n"/>
@@ -4996,11 +5022,20 @@
       <c r="F58" s="10" t="n"/>
       <c r="G58" s="10" t="n"/>
     </row>
+    <row r="59">
+      <c r="A59" s="11" t="n"/>
+      <c r="B59" s="11" t="n"/>
+      <c r="C59" s="11" t="n"/>
+      <c r="D59" s="11" t="n"/>
+      <c r="E59" s="11" t="n"/>
+      <c r="F59" s="11" t="n"/>
+      <c r="G59" s="11" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F58">
+  <conditionalFormatting sqref="F5:F59">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>F5="Done"</formula>
     </cfRule>
@@ -5014,7 +5049,7 @@
       <formula>F5="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E58">
+  <conditionalFormatting sqref="E5:E59">
     <cfRule type="expression" priority="5" dxfId="3">
       <formula>E5="P0"</formula>
     </cfRule>
@@ -5029,10 +5064,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="F5:F58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F5:F59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Done,In Progress,Not Started,Blocked"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2,P3"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>